<commit_message>
Refine dashboard section layout and typography
</commit_message>
<xml_diff>
--- a/mapping data.xlsx
+++ b/mapping data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranthihoanganh/Downloads/Customer Intelligence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7BE66284-9706-F24A-B65F-149293914298}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9FA7DDE-4314-6B4B-B3A1-3D07E9D80247}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16140" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="110">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="119">
   <si>
     <t>Overview</t>
   </si>
@@ -698,6 +698,9 @@
     <t>Theo đóng góp doanh thu</t>
   </si>
   <si>
+    <t>% đóng góp</t>
+  </si>
+  <si>
     <t>Theo thời điểm mua hàng</t>
   </si>
   <si>
@@ -945,6 +948,30 @@
   </si>
   <si>
     <t>% đóng góp theo số lưọng đơn</t>
+  </si>
+  <si>
+    <t>Phân khúc khách hàng</t>
+  </si>
+  <si>
+    <t>Ngủ đông</t>
+  </si>
+  <si>
+    <t>Khách thường</t>
+  </si>
+  <si>
+    <t>Tiềm năng</t>
+  </si>
+  <si>
+    <t>Nguy cơ rời bỏ</t>
+  </si>
+  <si>
+    <t>VIP</t>
+  </si>
+  <si>
+    <t>Tổng số khách hàng</t>
+  </si>
+  <si>
+    <t>% số khách hàng</t>
   </si>
 </sst>
 </file>
@@ -2185,7 +2212,7 @@
     </row>
     <row r="27" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A27" s="14" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B27" s="2">
         <v>74.08</v>
@@ -2219,7 +2246,7 @@
     </row>
     <row r="28" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A28" s="14" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B28" s="2">
         <v>69.11</v>
@@ -2253,7 +2280,7 @@
     </row>
     <row r="29" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A29" s="10" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" s="11"/>
       <c r="C29" s="11"/>
@@ -2283,7 +2310,7 @@
     </row>
     <row r="30" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A30" s="12" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" s="11"/>
       <c r="C30" s="11"/>
@@ -2313,13 +2340,13 @@
     </row>
     <row r="31" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A31" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -2347,10 +2374,10 @@
     </row>
     <row r="32" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A32" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C32" s="4">
         <v>22</v>
@@ -2381,10 +2408,10 @@
     </row>
     <row r="33" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A33" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C33" s="4">
         <v>7</v>
@@ -2415,10 +2442,10 @@
     </row>
     <row r="34" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A34" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C34" s="4">
         <v>10</v>
@@ -2449,10 +2476,10 @@
     </row>
     <row r="35" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A35" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C35" s="4">
         <v>7</v>
@@ -2483,10 +2510,10 @@
     </row>
     <row r="36" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A36" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C36" s="4">
         <v>12</v>
@@ -2517,10 +2544,10 @@
     </row>
     <row r="37" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A37" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C37" s="4">
         <v>10</v>
@@ -2551,10 +2578,10 @@
     </row>
     <row r="38" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A38" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C38" s="4">
         <v>26</v>
@@ -2585,10 +2612,10 @@
     </row>
     <row r="39" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A39" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C39" s="4">
         <v>14</v>
@@ -2619,10 +2646,10 @@
     </row>
     <row r="40" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A40" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C40" s="4">
         <v>10</v>
@@ -2653,10 +2680,10 @@
     </row>
     <row r="41" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A41" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C41" s="4">
         <v>17</v>
@@ -2687,10 +2714,10 @@
     </row>
     <row r="42" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A42" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C42" s="4">
         <v>11</v>
@@ -2721,10 +2748,10 @@
     </row>
     <row r="43" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A43" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C43" s="4">
         <v>11</v>
@@ -2755,10 +2782,10 @@
     </row>
     <row r="44" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A44" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C44" s="4">
         <v>30</v>
@@ -2789,10 +2816,10 @@
     </row>
     <row r="45" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A45" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B45" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C45" s="4">
         <v>25</v>
@@ -2823,10 +2850,10 @@
     </row>
     <row r="46" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A46" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B46" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C46" s="4">
         <v>6</v>
@@ -2857,10 +2884,10 @@
     </row>
     <row r="47" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A47" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B47" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C47" s="4">
         <v>10</v>
@@ -2891,10 +2918,10 @@
     </row>
     <row r="48" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A48" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B48" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C48" s="4">
         <v>11</v>
@@ -2925,10 +2952,10 @@
     </row>
     <row r="49" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A49" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C49" s="4">
         <v>5</v>
@@ -2959,10 +2986,10 @@
     </row>
     <row r="50" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A50" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B50" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C50" s="4">
         <v>22</v>
@@ -2993,10 +3020,10 @@
     </row>
     <row r="51" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A51" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B51" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C51" s="4">
         <v>7</v>
@@ -3027,10 +3054,10 @@
     </row>
     <row r="52" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A52" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B52" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C52" s="4">
         <v>9</v>
@@ -3061,10 +3088,10 @@
     </row>
     <row r="53" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A53" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C53" s="4">
         <v>13</v>
@@ -3095,10 +3122,10 @@
     </row>
     <row r="54" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A54" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B54" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C54" s="4">
         <v>5</v>
@@ -3129,10 +3156,10 @@
     </row>
     <row r="55" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A55" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B55" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C55" s="4">
         <v>8</v>
@@ -3163,10 +3190,10 @@
     </row>
     <row r="56" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A56" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B56" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C56" s="4">
         <v>30</v>
@@ -3197,10 +3224,10 @@
     </row>
     <row r="57" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A57" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B57" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C57" s="4">
         <v>15</v>
@@ -3231,10 +3258,10 @@
     </row>
     <row r="58" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A58" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C58" s="4">
         <v>10</v>
@@ -3265,10 +3292,10 @@
     </row>
     <row r="59" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A59" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B59" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C59" s="4">
         <v>15</v>
@@ -3299,10 +3326,10 @@
     </row>
     <row r="60" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A60" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B60" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C60" s="4">
         <v>4</v>
@@ -3333,10 +3360,10 @@
     </row>
     <row r="61" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A61" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B61" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C61" s="4">
         <v>6</v>
@@ -3367,10 +3394,10 @@
     </row>
     <row r="62" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A62" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B62" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C62" s="4">
         <v>19</v>
@@ -3401,10 +3428,10 @@
     </row>
     <row r="63" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A63" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B63" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C63" s="4">
         <v>10</v>
@@ -3435,10 +3462,10 @@
     </row>
     <row r="64" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A64" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C64" s="4">
         <v>6</v>
@@ -3469,10 +3496,10 @@
     </row>
     <row r="65" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A65" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C65" s="4">
         <v>11</v>
@@ -3503,10 +3530,10 @@
     </row>
     <row r="66" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A66" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B66" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C66" s="4">
         <v>12</v>
@@ -3537,10 +3564,10 @@
     </row>
     <row r="67" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A67" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B67" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C67" s="4">
         <v>7</v>
@@ -3571,10 +3598,10 @@
     </row>
     <row r="68" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A68" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B68" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C68" s="4">
         <v>24</v>
@@ -3605,10 +3632,10 @@
     </row>
     <row r="69" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A69" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B69" s="2" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C69" s="4">
         <v>10</v>
@@ -3639,10 +3666,10 @@
     </row>
     <row r="70" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A70" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B70" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C70" s="4">
         <v>19</v>
@@ -3673,10 +3700,10 @@
     </row>
     <row r="71" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A71" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C71" s="4">
         <v>8</v>
@@ -3707,10 +3734,10 @@
     </row>
     <row r="72" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A72" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B72" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C72" s="4">
         <v>11</v>
@@ -3741,10 +3768,10 @@
     </row>
     <row r="73" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A73" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B73" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C73" s="4">
         <v>5</v>
@@ -3805,10 +3832,10 @@
     </row>
     <row r="75" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A75" s="2" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="B75" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C75" s="2"/>
       <c r="D75" s="2"/>
@@ -3837,7 +3864,7 @@
     </row>
     <row r="76" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A76" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B76" s="4">
         <v>68</v>
@@ -3869,7 +3896,7 @@
     </row>
     <row r="77" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A77" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B77" s="4">
         <v>89</v>
@@ -3901,7 +3928,7 @@
     </row>
     <row r="78" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A78" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B78" s="4">
         <v>87</v>
@@ -3933,7 +3960,7 @@
     </row>
     <row r="79" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A79" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="B79" s="4">
         <v>64</v>
@@ -3965,7 +3992,7 @@
     </row>
     <row r="80" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A80" s="2" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B80" s="4">
         <v>80</v>
@@ -3997,7 +4024,7 @@
     </row>
     <row r="81" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A81" s="2" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B81" s="4">
         <v>65</v>
@@ -4029,7 +4056,7 @@
     </row>
     <row r="82" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A82" s="2" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B82" s="4">
         <v>77</v>
@@ -4061,7 +4088,7 @@
     </row>
     <row r="83" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A83" s="10" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B83" s="11"/>
       <c r="C83" s="11"/>
@@ -4091,13 +4118,13 @@
     </row>
     <row r="84" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A84" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B84" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D84" s="2"/>
       <c r="E84" s="2"/>
@@ -4125,7 +4152,7 @@
     </row>
     <row r="85" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A85" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B85" s="4">
         <v>29</v>
@@ -4158,7 +4185,7 @@
     </row>
     <row r="86" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A86" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B86" s="4">
         <v>19</v>
@@ -4191,7 +4218,7 @@
     </row>
     <row r="87" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A87" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B87" s="4">
         <v>13</v>
@@ -4224,7 +4251,7 @@
     </row>
     <row r="88" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A88" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B88" s="4">
         <v>10</v>
@@ -4257,7 +4284,7 @@
     </row>
     <row r="89" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A89" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B89" s="4">
         <v>9</v>
@@ -4290,7 +4317,7 @@
     </row>
     <row r="90" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A90" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B90" s="4">
         <v>7</v>
@@ -4323,7 +4350,7 @@
     </row>
     <row r="91" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A91" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B91" s="4">
         <v>7</v>
@@ -4356,7 +4383,7 @@
     </row>
     <row r="92" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A92" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B92" s="4">
         <v>6</v>
@@ -4389,7 +4416,7 @@
     </row>
     <row r="93" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A93" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B93" s="4">
         <v>3</v>
@@ -4422,7 +4449,7 @@
     </row>
     <row r="94" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A94" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B94" s="4">
         <v>2</v>
@@ -4455,7 +4482,7 @@
     </row>
     <row r="95" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A95" s="2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B95" s="4">
         <v>1</v>
@@ -4549,10 +4576,10 @@
     <row r="98" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A98" s="3"/>
       <c r="B98" s="5" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C98" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D98" s="2"/>
       <c r="E98" s="2"/>
@@ -4580,7 +4607,7 @@
     </row>
     <row r="99" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A99" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B99" s="4">
         <v>80</v>
@@ -4615,7 +4642,7 @@
     </row>
     <row r="100" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A100" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B100" s="4">
         <v>137</v>
@@ -4650,7 +4677,7 @@
     </row>
     <row r="101" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A101" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B101" s="4">
         <v>30</v>
@@ -4686,10 +4713,10 @@
     <row r="102" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A102" s="2"/>
       <c r="B102" s="5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C102" s="5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D102" s="2"/>
       <c r="E102" s="2"/>
@@ -4717,13 +4744,13 @@
     </row>
     <row r="103" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A103" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B103" s="4">
         <v>11545411</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D103" s="2"/>
       <c r="E103" s="2"/>
@@ -4751,13 +4778,13 @@
     </row>
     <row r="104" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A104" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B104" s="4">
         <v>13507069</v>
       </c>
       <c r="C104" s="2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D104" s="2"/>
       <c r="E104" s="2"/>
@@ -4785,13 +4812,13 @@
     </row>
     <row r="105" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A105" s="2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B105" s="4">
         <v>5034040</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D105" s="2"/>
       <c r="E105" s="2"/>
@@ -4819,7 +4846,7 @@
     </row>
     <row r="106" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A106" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B106" s="11"/>
       <c r="C106" s="11"/>
@@ -4850,20 +4877,20 @@
     <row r="107" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A107" s="2"/>
       <c r="B107" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C107" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D107" s="2"/>
       <c r="E107" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F107" s="2" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="G107" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="H107" s="2"/>
       <c r="I107" s="2"/>
@@ -4890,13 +4917,13 @@
         <v>1</v>
       </c>
       <c r="B108" s="2" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C108" s="9">
         <v>20140942183</v>
       </c>
       <c r="D108" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E108" s="4">
         <v>7</v>
@@ -4930,13 +4957,13 @@
         <v>2</v>
       </c>
       <c r="B109" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C109" s="9">
         <v>15484234913</v>
       </c>
       <c r="D109" s="4" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E109" s="4">
         <v>7</v>
@@ -4970,13 +4997,13 @@
         <v>3</v>
       </c>
       <c r="B110" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C110" s="9">
         <v>29233346058</v>
       </c>
       <c r="D110" s="4" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E110" s="4">
         <v>6</v>
@@ -5010,13 +5037,13 @@
         <v>4</v>
       </c>
       <c r="B111" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C111" s="9">
         <v>15484234913</v>
       </c>
       <c r="D111" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E111" s="4">
         <v>5</v>
@@ -5050,7 +5077,7 @@
         <v>5</v>
       </c>
       <c r="B112" s="2" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C112" s="9">
         <v>49813936807</v>
@@ -5088,13 +5115,13 @@
         <v>6</v>
       </c>
       <c r="B113" s="2" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C113" s="9">
         <v>20540949887</v>
       </c>
       <c r="D113" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E113" s="4">
         <v>4</v>
@@ -5128,7 +5155,7 @@
         <v>7</v>
       </c>
       <c r="B114" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C114" s="9">
         <v>44552142483</v>
@@ -5166,7 +5193,7 @@
         <v>8</v>
       </c>
       <c r="B115" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C115" s="9">
         <v>52563959751</v>
@@ -5204,13 +5231,13 @@
         <v>9</v>
       </c>
       <c r="B116" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C116" s="9">
         <v>57313958189</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E116" s="4">
         <v>1</v>
@@ -5244,13 +5271,13 @@
         <v>10</v>
       </c>
       <c r="B117" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C117" s="9">
         <v>25893057187</v>
       </c>
       <c r="D117" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E117" s="4">
         <v>1</v>
@@ -5282,7 +5309,7 @@
     <row r="118" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A118" s="4"/>
       <c r="B118" s="2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C118" s="9"/>
       <c r="D118" s="4"/>
@@ -5312,7 +5339,7 @@
         <v>1</v>
       </c>
       <c r="B119" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C119" s="9">
         <v>15584241449</v>
@@ -5350,7 +5377,7 @@
         <v>2</v>
       </c>
       <c r="B120" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C120" s="9">
         <v>15484234913</v>
@@ -5388,7 +5415,7 @@
         <v>3</v>
       </c>
       <c r="B121" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C121" s="9">
         <v>24956187823</v>
@@ -5426,7 +5453,7 @@
         <v>4</v>
       </c>
       <c r="B122" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C122" s="9">
         <v>15084234863</v>
@@ -5464,7 +5491,7 @@
         <v>5</v>
       </c>
       <c r="B123" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C123" s="9">
         <v>16167874509</v>
@@ -5502,7 +5529,7 @@
         <v>6</v>
       </c>
       <c r="B124" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C124" s="9">
         <v>24616846046</v>
@@ -5540,7 +5567,7 @@
         <v>7</v>
       </c>
       <c r="B125" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C125" s="9">
         <v>12892358205</v>
@@ -5578,7 +5605,7 @@
         <v>8</v>
       </c>
       <c r="B126" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C126" s="9">
         <v>16067874699</v>
@@ -5616,7 +5643,7 @@
         <v>9</v>
       </c>
       <c r="B127" s="2" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C127" s="9">
         <v>16067874699</v>
@@ -5654,7 +5681,7 @@
         <v>10</v>
       </c>
       <c r="B128" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C128" s="9">
         <v>15084234863</v>
@@ -5689,7 +5716,7 @@
     </row>
     <row r="129" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A129" s="12" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="B129" s="11"/>
       <c r="C129" s="11"/>
@@ -5720,19 +5747,19 @@
     <row r="130" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A130" s="2"/>
       <c r="B130" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C130" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="D130" s="2" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E130" s="2" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="F130" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="G130" s="2"/>
       <c r="H130" s="2"/>
@@ -5763,13 +5790,13 @@
         <v>29233346058</v>
       </c>
       <c r="C131" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="D131" s="9">
         <v>42801105610</v>
       </c>
       <c r="E131" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F131" s="4">
         <v>3</v>
@@ -5803,13 +5830,13 @@
         <v>24956187823</v>
       </c>
       <c r="C132" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="D132" s="9">
         <v>42801105610</v>
       </c>
       <c r="E132" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F132" s="4">
         <v>2</v>
@@ -5843,13 +5870,13 @@
         <v>26580532173</v>
       </c>
       <c r="C133" s="4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="D133" s="9">
         <v>42801105610</v>
       </c>
       <c r="E133" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F133" s="4">
         <v>2</v>
@@ -5883,13 +5910,13 @@
         <v>15284234921</v>
       </c>
       <c r="C134" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="D134" s="9">
         <v>24616846046</v>
       </c>
       <c r="E134" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="F134" s="4">
         <v>2</v>
@@ -5923,13 +5950,13 @@
         <v>24956187823</v>
       </c>
       <c r="C135" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D135" s="9">
         <v>42801105610</v>
       </c>
       <c r="E135" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F135" s="4">
         <v>2</v>
@@ -6012,7 +6039,9 @@
       <c r="Z137" s="2"/>
     </row>
     <row r="138" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A138" s="2"/>
+      <c r="A138" s="14" t="s">
+        <v>111</v>
+      </c>
       <c r="B138" s="2"/>
       <c r="C138" s="2"/>
       <c r="D138" s="2"/>
@@ -6040,11 +6069,21 @@
       <c r="Z138" s="2"/>
     </row>
     <row r="139" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A139" s="2"/>
-      <c r="B139" s="2"/>
-      <c r="C139" s="2"/>
-      <c r="D139" s="2"/>
-      <c r="E139" s="2"/>
+      <c r="A139" s="14" t="s">
+        <v>111</v>
+      </c>
+      <c r="B139" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C139" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="D139" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="E139" s="14" t="s">
+        <v>27</v>
+      </c>
       <c r="F139" s="2"/>
       <c r="G139" s="2"/>
       <c r="H139" s="2"/>
@@ -6068,12 +6107,21 @@
       <c r="Z139" s="2"/>
     </row>
     <row r="140" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A140" s="2"/>
-      <c r="B140" s="2"/>
-      <c r="C140" s="2"/>
-      <c r="D140" s="2"/>
-      <c r="E140" s="2"/>
-      <c r="F140" s="2"/>
+      <c r="A140" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="B140" s="2">
+        <v>192</v>
+      </c>
+      <c r="C140" s="2">
+        <v>39.340000000000003</v>
+      </c>
+      <c r="D140" s="2">
+        <v>22872121</v>
+      </c>
+      <c r="E140" s="2">
+        <v>39.659999999999997</v>
+      </c>
       <c r="G140" s="2"/>
       <c r="H140" s="2"/>
       <c r="I140" s="2"/>
@@ -6096,12 +6144,21 @@
       <c r="Z140" s="2"/>
     </row>
     <row r="141" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A141" s="2"/>
-      <c r="B141" s="2"/>
-      <c r="C141" s="2"/>
-      <c r="D141" s="2"/>
-      <c r="E141" s="2"/>
-      <c r="F141" s="2"/>
+      <c r="A141" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B141" s="2">
+        <v>179</v>
+      </c>
+      <c r="C141" s="2">
+        <v>36.68</v>
+      </c>
+      <c r="D141" s="2">
+        <v>18368331</v>
+      </c>
+      <c r="E141" s="2">
+        <v>31.85</v>
+      </c>
       <c r="G141" s="2"/>
       <c r="H141" s="2"/>
       <c r="I141" s="2"/>
@@ -6124,12 +6181,21 @@
       <c r="Z141" s="2"/>
     </row>
     <row r="142" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A142" s="2"/>
-      <c r="B142" s="2"/>
-      <c r="C142" s="2"/>
-      <c r="D142" s="2"/>
-      <c r="E142" s="2"/>
-      <c r="F142" s="2"/>
+      <c r="A142" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B142" s="2">
+        <v>98</v>
+      </c>
+      <c r="C142" s="2">
+        <v>20.079999999999998</v>
+      </c>
+      <c r="D142" s="2">
+        <v>11159748</v>
+      </c>
+      <c r="E142" s="2">
+        <v>19.350000000000001</v>
+      </c>
       <c r="G142" s="2"/>
       <c r="H142" s="2"/>
       <c r="I142" s="2"/>
@@ -6152,12 +6218,21 @@
       <c r="Z142" s="2"/>
     </row>
     <row r="143" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A143" s="2"/>
-      <c r="B143" s="2"/>
-      <c r="C143" s="2"/>
-      <c r="D143" s="2"/>
-      <c r="E143" s="2"/>
-      <c r="F143" s="2"/>
+      <c r="A143" s="2" t="s">
+        <v>114</v>
+      </c>
+      <c r="B143" s="2">
+        <v>16</v>
+      </c>
+      <c r="C143" s="2">
+        <v>3.28</v>
+      </c>
+      <c r="D143" s="2">
+        <v>3269197</v>
+      </c>
+      <c r="E143" s="2">
+        <v>5.67</v>
+      </c>
       <c r="G143" s="2"/>
       <c r="H143" s="2"/>
       <c r="I143" s="2"/>
@@ -6180,12 +6255,21 @@
       <c r="Z143" s="2"/>
     </row>
     <row r="144" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A144" s="2"/>
-      <c r="B144" s="2"/>
-      <c r="C144" s="2"/>
-      <c r="D144" s="2"/>
-      <c r="E144" s="2"/>
-      <c r="F144" s="2"/>
+      <c r="A144" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B144" s="2">
+        <v>2</v>
+      </c>
+      <c r="C144" s="2">
+        <v>0.41</v>
+      </c>
+      <c r="D144" s="2">
+        <v>1113299</v>
+      </c>
+      <c r="E144" s="2">
+        <v>1.93</v>
+      </c>
       <c r="G144" s="2"/>
       <c r="H144" s="2"/>
       <c r="I144" s="2"/>
@@ -6208,12 +6292,21 @@
       <c r="Z144" s="2"/>
     </row>
     <row r="145" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A145" s="2"/>
-      <c r="B145" s="2"/>
-      <c r="C145" s="2"/>
-      <c r="D145" s="2"/>
-      <c r="E145" s="2"/>
-      <c r="F145" s="2"/>
+      <c r="A145" s="2" t="s">
+        <v>116</v>
+      </c>
+      <c r="B145" s="2">
+        <v>1</v>
+      </c>
+      <c r="C145" s="2">
+        <v>0.2</v>
+      </c>
+      <c r="D145" s="2">
+        <v>888720</v>
+      </c>
+      <c r="E145" s="2">
+        <v>1.54</v>
+      </c>
       <c r="G145" s="2"/>
       <c r="H145" s="2"/>
       <c r="I145" s="2"/>

</xml_diff>

<commit_message>
Update Customer Intelligence with latest customer data
</commit_message>
<xml_diff>
--- a/mapping data.xlsx
+++ b/mapping data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranthihoanganh/Downloads/Customer Intelligence/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E255FA61-E593-3A44-B87A-92016D603734}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4AAB8B3-7924-8341-A246-195DEFF3AACE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="16100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="484" uniqueCount="207">
   <si>
     <t>Overview</t>
   </si>
@@ -1045,6 +1045,198 @@
   <si>
     <t>480.5M</t>
   </si>
+  <si>
+    <t>order_date</t>
+  </si>
+  <si>
+    <t>new_customers</t>
+  </si>
+  <si>
+    <t>existing_customers</t>
+  </si>
+  <si>
+    <t>total_customers</t>
+  </si>
+  <si>
+    <t>new_customer_orders</t>
+  </si>
+  <si>
+    <t>existing_customer_orders</t>
+  </si>
+  <si>
+    <t>total_orders</t>
+  </si>
+  <si>
+    <t>new_customer_revenue</t>
+  </si>
+  <si>
+    <t>existing_customer_revenue</t>
+  </si>
+  <si>
+    <t>total_revenue</t>
+  </si>
+  <si>
+    <t>Khách mới, khách cũ</t>
+  </si>
+  <si>
+    <t>cancel_reason</t>
+  </si>
+  <si>
+    <t>cancelled_orders</t>
+  </si>
+  <si>
+    <t>cancelled_order_rate_percent</t>
+  </si>
+  <si>
+    <t>lost_revenue</t>
+  </si>
+  <si>
+    <t>lost_revenue_rate_percent</t>
+  </si>
+  <si>
+    <t>customer_segment</t>
+  </si>
+  <si>
+    <t>customer_rate_percent</t>
+  </si>
+  <si>
+    <t>revenue_contribution_percent</t>
+  </si>
+  <si>
+    <t>avg_recency_days</t>
+  </si>
+  <si>
+    <t>avg_frequency</t>
+  </si>
+  <si>
+    <t>avg_monetary</t>
+  </si>
+  <si>
+    <t>Potential</t>
+  </si>
+  <si>
+    <t>Customer segmentation</t>
+  </si>
+  <si>
+    <t>snapshot_date</t>
+  </si>
+  <si>
+    <t>new_customer_top_3_products</t>
+  </si>
+  <si>
+    <t>existing_customer_top_3_products</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 4}, {"rank": 2, "orders": 3, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "1 hộp lẻ", "quantity_sold": 3}, {"rank": 3, "orders": 3, "item_id": "20140942183", "item_name": "Combo 2 Hủ Kẹo Cà Phê Sữa Mayora Kopiko 560G", "model_name": "Combo 2", "quantity_sold": 3}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "combo 2 hộp", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "20140942183", "item_name": "Combo 2 Hủ Kẹo Cà Phê Sữa Mayora Kopiko 560G", "model_name": "Combo 2", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 8, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CALCHESE 153G 7/2026", "quantity_sold": 8}, {"rank": 2, "orders": 3, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 4}, {"rank": 3, "orders": 3, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 3}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "46451334830", "item_name": "Bánh Quế Xốp Kem Socola Mayora Go Choco Rollz 375G", "model_name": "1 HỘP", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "26580532173", "item_name": "Bánh Quy Sữa Mới Mayora D-Maxx Marie - Hộp Giấy 308G (14 Gói X 22G)", "model_name": "308G", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "47601348595", "item_name": "Bánh Xốp Mayora Superstar 375G (30 Thanh X12.5G)", "model_name": "1 HỘP", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "15084234863", "item_name": "Kẹo Cà Phê Sữa Mayora Kopiko 140G", "model_name": "KẸO CÀ PHÊ ĐEN", "quantity_sold": 5}, {"rank": 2, "orders": 3, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "COMBO 5 GÓI", "quantity_sold": 4}, {"rank": 3, "orders": 3, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 4}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "46451334830", "item_name": "Bánh Quế Xốp Kem Socola Mayora Go Choco Rollz 375G", "model_name": "2 HỘP", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "42801105610", "item_name": "Bánh Quy Bơ &amp; Cacao Mayora Danisa Abbracci Hộp 168G", "model_name": "1 hộp lẻ", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CALCHESE 153G 7/2026", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 3, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 3}, {"rank": 2, "orders": 2, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 2}, {"rank": 3, "orders": 1, "item_id": "46451334830", "item_name": "Bánh Quế Xốp Kem Socola Mayora Go Choco Rollz 375G", "model_name": "2 HỘP", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CAL CHEESE 200G", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "16067874699", "item_name": "Kẹo Mayora The Fres Barley 150G", "model_name": "KẸO XANH LÁ", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "16167874509", "item_name": "Bánh Quy Bơ Mayora Danisa 681G", "model_name": "", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "16167874390", "item_name": "Bánh Quy Vị Cà Phê Mayora Coffee Joy 156G", "model_name": "2hộp156g HSD 11/2026", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "16067874699", "item_name": "Kẹo Mayora The Fres Barley 150G", "model_name": "KẸO ME TAMARIN", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "combo 2 hộp", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "15184234867", "item_name": "Bánh Quy Vị Cà Phê Mayora Coffee Joy 312G", "model_name": "Hộp Coffe joy 312G", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "COMBO 2 GÓI", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "51063922408", "item_name": "Combo Văn Phòng Kopiko", "model_name": "Kẹo Đen + macchiato", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "51063922408", "item_name": "Combo Văn Phòng Kopiko", "model_name": "Kẹo Sữa + macchiato", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "51957402000", "item_name": "Bánh Quy Bơ Mayora Danisa 72G", "model_name": "2 HỘP", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[]</t>
+  </si>
+  <si>
+    <t>Khách mới, khách cũ + Top 3</t>
+  </si>
+  <si>
+    <t>Phân khúc + Top 3</t>
+  </si>
+  <si>
+    <t>top_3_products</t>
+  </si>
+  <si>
+    <t>Top Buyers</t>
+  </si>
+  <si>
+    <t>Big Spenders</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 4, "item_id": "20140942183", "item_name": "Combo 2 Hủ Kẹo Cà Phê Sữa Mayora Kopiko 560G", "model_name": "Combo 2", "quantity_sold": 4}, {"rank": 2, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 4}, {"rank": 3, "orders": 3, "item_id": "45602582884", "item_name": "( Quà Tặng Livestream) Phiên Live Danisa", "model_name": "1 GÓI", "quantity_sold": 3}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "1 hộp lẻ", "quantity_sold": 2}, {"rank": 2, "orders": 2, "item_id": "15084234863", "item_name": "Kẹo Cà Phê Sữa Mayora Kopiko 140G", "model_name": "KẸO CÀ PHÊ ĐEN", "quantity_sold": 2}, {"rank": 3, "orders": 1, "item_id": "16167874390", "item_name": "Bánh Quy Vị Cà Phê Mayora Coffee Joy 156G", "model_name": "1hộp156g HSD11/2026", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>Occasional Buyers</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "42801105610", "item_name": "Bánh Quy Bơ &amp; Cacao Mayora Danisa Abbracci Hộp 168G", "model_name": "1 hộp lẻ", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "1 hộp lẻ", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 8, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CALCHESE 153G 7/2026", "quantity_sold": 8}, {"rank": 2, "orders": 2, "item_id": "16167874509", "item_name": "Bánh Quy Bơ Mayora Danisa 681G", "model_name": "", "quantity_sold": 2}, {"rank": 3, "orders": 2, "item_id": "47601348595", "item_name": "Bánh Xốp Mayora Superstar 375G (30 Thanh X12.5G)", "model_name": "1 HỘP", "quantity_sold": 2}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 3, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 3}, {"rank": 2, "orders": 2, "item_id": "12892358205", "item_name": "Kẹo Cà Phê Sữa Mayora Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 2}, {"rank": 3, "orders": 1, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "WAFELLO 210G", "quantity_sold": 2}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 2}, {"rank": 2, "orders": 2, "item_id": "20140942183", "item_name": "Combo 2 Hủ Kẹo Cà Phê Sữa Mayora Kopiko 560G", "model_name": "Combo 2", "quantity_sold": 2}, {"rank": 3, "orders": 1, "item_id": "42801105610", "item_name": "Bánh Quy Bơ &amp; Cacao Mayora Danisa Abbracci Hộp 168G", "model_name": "combo 2 hộp", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 4, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "COMBO 5 GÓI", "quantity_sold": 5}, {"rank": 2, "orders": 2, "item_id": "46451334830", "item_name": "Bánh Quế Xốp Kem Socola Mayora Go Choco Rollz 375G", "model_name": "2 HỘP", "quantity_sold": 2}, {"rank": 3, "orders": 2, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CALCHESE 153G 7/2026", "quantity_sold": 2}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "49813936807", "item_name": "Combo Best Seller", "model_name": "", "quantity_sold": 2}, {"rank": 2, "orders": 2, "item_id": "15584241449", "item_name": "Kẹo Mayora Cà Phê Kopiko 560G", "model_name": "1 hộp", "quantity_sold": 2}, {"rank": 3, "orders": 1, "item_id": "16067874699", "item_name": "Kẹo Mayora The Fres Barley 150G", "model_name": "KẸO XANH LÁ", "quantity_sold": 2}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "15084234863", "item_name": "Kẹo Cà Phê Sữa Mayora Kopiko 140G", "model_name": "KẸO CÀ PHÊ ĐEN", "quantity_sold": 6}, {"rank": 2, "orders": 1, "item_id": "26580532173", "item_name": "Bánh Quy Sữa Mới Mayora D-Maxx Marie - Hộp Giấy 308G (14 Gói X 22G)", "model_name": "220G", "quantity_sold": 3}, {"rank": 3, "orders": 2, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 2}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "46451334830", "item_name": "Bánh Quế Xốp Kem Socola Mayora Go Choco Rollz 375G", "model_name": "2 HỘP", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "16167874509", "item_name": "Bánh Quy Bơ Mayora Danisa 681G", "model_name": "", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "24616846046", "item_name": "Bánh Xốp Mayora Wafello Chocolate 210G", "model_name": "CAL CHEESE 200G", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "20540949887", "item_name": "Combo 2 Kẹo Cà Phê Sữa Mayora Kopiko 135G", "model_name": "2 gói cà phê sữa", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 2, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "COMBO 5 GÓI", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "16167874509", "item_name": "Bánh Quy Bơ Mayora Danisa 681G", "model_name": "", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "24956187823", "item_name": "Bánh Quy Bơ Mayora Danisa 200G", "model_name": "", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "16167874390", "item_name": "Bánh Quy Vị Cà Phê Mayora Coffee Joy 156G", "model_name": "2hộp156g HSD 11/2026", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "1 GÓI", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "16067874699", "item_name": "Kẹo Mayora The Fres Barley 150G", "model_name": "KẸO ME TAMARIN", "quantity_sold": 2}, {"rank": 2, "orders": 1, "item_id": "16167874509", "item_name": "Bánh Quy Bơ Mayora Danisa 681G", "model_name": "", "quantity_sold": 1}, {"rank": 3, "orders": 1, "item_id": "29233346058", "item_name": "Bánh Quy Mayora Danisa Chocofello 150G", "model_name": "combo 2 hộp", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "15484234913", "item_name": "Cà Phê Sữa Hòa Tan Mayora Kopiko Macchiato 400G", "model_name": "COMBO 2 GÓI", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "51957402000", "item_name": "Bánh Quy Bơ Mayora Danisa 72G", "model_name": "2 HỘP", "quantity_sold": 1}, {"rank": 2, "orders": 1, "item_id": "51063922408", "item_name": "Combo Văn Phòng Kopiko", "model_name": "Kẹo Đen + macchiato", "quantity_sold": 1}]</t>
+  </si>
+  <si>
+    <t>[{"rank": 1, "orders": 1, "item_id": "51063922408", "item_name": "Combo Văn Phòng Kopiko", "model_name": "Kẹo Sữa + macchiato", "quantity_sold": 1}]</t>
+  </si>
 </sst>
 </file>
 
@@ -1054,7 +1246,7 @@
     <numFmt numFmtId="164" formatCode="d/m/yyyy"/>
     <numFmt numFmtId="165" formatCode="dd\.mm"/>
   </numFmts>
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="10" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1106,6 +1298,19 @@
       <name val="Times New Roman"/>
       <family val="1"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica Neue"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1127,7 +1332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1144,20 +1349,29 @@
     <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="10" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="9" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="39" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="39" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="39" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="39" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1433,22 +1647,22 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:Z1006"/>
+  <dimension ref="A1:Z1007"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="26" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A1" s="15" t="s">
+      <c r="A1" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="C1" s="13"/>
-      <c r="D1" s="13"/>
-      <c r="E1" s="13"/>
-      <c r="F1" s="13"/>
-      <c r="G1" s="13"/>
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21"/>
+      <c r="G1" s="21"/>
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
@@ -1470,14 +1684,14 @@
       <c r="Z1" s="2"/>
     </row>
     <row r="2" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="13"/>
-      <c r="C2" s="13"/>
-      <c r="D2" s="13"/>
-      <c r="E2" s="13"/>
-      <c r="F2" s="13"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
@@ -1580,11 +1794,11 @@
       <c r="Z4" s="2"/>
     </row>
     <row r="5" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="13"/>
-      <c r="C5" s="13"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
       <c r="D5" s="2"/>
       <c r="E5" s="2"/>
       <c r="F5" s="2"/>
@@ -2252,11 +2466,11 @@
       <c r="Z24" s="2"/>
     </row>
     <row r="25" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A25" s="14" t="s">
+      <c r="A25" s="20" t="s">
         <v>26</v>
       </c>
-      <c r="B25" s="13"/>
-      <c r="C25" s="13"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
@@ -2382,11 +2596,11 @@
       <c r="Z28" s="2"/>
     </row>
     <row r="29" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B29" s="13"/>
-      <c r="C29" s="13"/>
+      <c r="B29" s="21"/>
+      <c r="C29" s="21"/>
       <c r="D29" s="2"/>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -2412,11 +2626,11 @@
       <c r="Z29" s="2"/>
     </row>
     <row r="30" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A30" s="14" t="s">
+      <c r="A30" s="20" t="s">
         <v>29</v>
       </c>
-      <c r="B30" s="13"/>
-      <c r="C30" s="13"/>
+      <c r="B30" s="21"/>
+      <c r="C30" s="21"/>
       <c r="D30" s="2"/>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
@@ -3904,11 +4118,11 @@
       <c r="Z73" s="2"/>
     </row>
     <row r="74" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A74" s="14" t="s">
+      <c r="A74" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="B74" s="13"/>
-      <c r="C74" s="13"/>
+      <c r="B74" s="21"/>
+      <c r="C74" s="21"/>
       <c r="D74" s="2"/>
       <c r="E74" s="2"/>
       <c r="F74" s="2"/>
@@ -4190,11 +4404,11 @@
       <c r="Z82" s="2"/>
     </row>
     <row r="83" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A83" s="12" t="s">
+      <c r="A83" s="24" t="s">
         <v>48</v>
       </c>
-      <c r="B83" s="13"/>
-      <c r="C83" s="13"/>
+      <c r="B83" s="21"/>
+      <c r="C83" s="21"/>
       <c r="D83" s="2"/>
       <c r="E83" s="2"/>
       <c r="F83" s="2"/>
@@ -4647,11 +4861,11 @@
       <c r="Z96" s="2"/>
     </row>
     <row r="97" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A97" s="12" t="s">
+      <c r="A97" s="24" t="s">
         <v>17</v>
       </c>
-      <c r="B97" s="13"/>
-      <c r="C97" s="13"/>
+      <c r="B97" s="21"/>
+      <c r="C97" s="21"/>
       <c r="D97" s="2"/>
       <c r="E97" s="2"/>
       <c r="F97" s="2"/>
@@ -4948,15 +5162,15 @@
       <c r="Z105" s="2"/>
     </row>
     <row r="106" spans="1:26" ht="13" x14ac:dyDescent="0.15">
-      <c r="A106" s="14" t="s">
+      <c r="A106" s="20" t="s">
         <v>70</v>
       </c>
-      <c r="B106" s="13"/>
-      <c r="C106" s="13"/>
-      <c r="D106" s="13"/>
-      <c r="E106" s="13"/>
-      <c r="F106" s="13"/>
-      <c r="G106" s="13"/>
+      <c r="B106" s="21"/>
+      <c r="C106" s="21"/>
+      <c r="D106" s="21"/>
+      <c r="E106" s="21"/>
+      <c r="F106" s="21"/>
+      <c r="G106" s="21"/>
       <c r="H106" s="2"/>
       <c r="I106" s="2"/>
       <c r="J106" s="2"/>
@@ -5818,15 +6032,15 @@
       <c r="Z128" s="2"/>
     </row>
     <row r="129" spans="1:26" ht="16.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A129" s="14" t="s">
+      <c r="A129" s="20" t="s">
         <v>97</v>
       </c>
-      <c r="B129" s="13"/>
-      <c r="C129" s="13"/>
-      <c r="D129" s="13"/>
-      <c r="E129" s="13"/>
-      <c r="F129" s="13"/>
-      <c r="G129" s="13"/>
+      <c r="B129" s="21"/>
+      <c r="C129" s="21"/>
+      <c r="D129" s="21"/>
+      <c r="E129" s="21"/>
+      <c r="F129" s="21"/>
+      <c r="G129" s="21"/>
       <c r="H129" s="2"/>
       <c r="I129" s="2"/>
       <c r="J129" s="2"/>
@@ -10099,14 +10313,14 @@
     </row>
     <row r="256" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A256" s="2"/>
-      <c r="B256" s="21" t="s">
+      <c r="B256" s="25" t="s">
         <v>125</v>
       </c>
-      <c r="C256" s="21"/>
-      <c r="D256" s="21"/>
-      <c r="E256" s="21"/>
-      <c r="F256" s="21"/>
-      <c r="G256" s="21"/>
+      <c r="C256" s="25"/>
+      <c r="D256" s="25"/>
+      <c r="E256" s="25"/>
+      <c r="F256" s="25"/>
+      <c r="G256" s="25"/>
       <c r="H256" s="2"/>
       <c r="I256" s="2"/>
       <c r="J256" s="2"/>
@@ -10129,22 +10343,22 @@
     </row>
     <row r="257" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A257" s="2"/>
-      <c r="B257" s="16" t="s">
+      <c r="B257" s="12" t="s">
         <v>125</v>
       </c>
-      <c r="C257" s="16" t="s">
+      <c r="C257" s="12" t="s">
         <v>126</v>
       </c>
-      <c r="D257" s="16" t="s">
+      <c r="D257" s="12" t="s">
         <v>127</v>
       </c>
-      <c r="E257" s="16" t="s">
+      <c r="E257" s="12" t="s">
         <v>128</v>
       </c>
-      <c r="F257" s="16" t="s">
+      <c r="F257" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="G257" s="16" t="s">
+      <c r="G257" s="12" t="s">
         <v>129</v>
       </c>
       <c r="H257" s="2"/>
@@ -10169,22 +10383,22 @@
     </row>
     <row r="258" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A258" s="2"/>
-      <c r="B258" s="16" t="s">
+      <c r="B258" s="12" t="s">
         <v>130</v>
       </c>
-      <c r="C258" s="17" t="s">
+      <c r="C258" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="D258" s="17">
+      <c r="D258" s="13">
         <v>486</v>
       </c>
-      <c r="E258" s="18">
+      <c r="E258" s="14">
         <v>0.48599999999999999</v>
       </c>
-      <c r="F258" s="17" t="s">
+      <c r="F258" s="13" t="s">
         <v>132</v>
       </c>
-      <c r="G258" s="18">
+      <c r="G258" s="14">
         <v>0.14199999999999999</v>
       </c>
       <c r="H258" s="2"/>
@@ -10209,22 +10423,22 @@
     </row>
     <row r="259" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A259" s="2"/>
-      <c r="B259" s="16" t="s">
+      <c r="B259" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="C259" s="17" t="s">
+      <c r="C259" s="13" t="s">
         <v>134</v>
       </c>
-      <c r="D259" s="17">
+      <c r="D259" s="13">
         <v>268</v>
       </c>
-      <c r="E259" s="18">
+      <c r="E259" s="14">
         <v>0.26800000000000002</v>
       </c>
-      <c r="F259" s="17" t="s">
+      <c r="F259" s="13" t="s">
         <v>135</v>
       </c>
-      <c r="G259" s="18">
+      <c r="G259" s="14">
         <v>0.23400000000000001</v>
       </c>
       <c r="H259" s="2"/>
@@ -10249,22 +10463,22 @@
     </row>
     <row r="260" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A260" s="2"/>
-      <c r="B260" s="16" t="s">
+      <c r="B260" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="C260" s="17" t="s">
+      <c r="C260" s="13" t="s">
         <v>137</v>
       </c>
-      <c r="D260" s="17">
+      <c r="D260" s="13">
         <v>151</v>
       </c>
-      <c r="E260" s="18">
+      <c r="E260" s="14">
         <v>0.151</v>
       </c>
-      <c r="F260" s="17" t="s">
+      <c r="F260" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="G260" s="18">
+      <c r="G260" s="14">
         <v>0.26600000000000001</v>
       </c>
       <c r="H260" s="2"/>
@@ -10289,22 +10503,22 @@
     </row>
     <row r="261" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A261" s="2"/>
-      <c r="B261" s="16" t="s">
+      <c r="B261" s="12" t="s">
         <v>116</v>
       </c>
-      <c r="C261" s="17" t="s">
+      <c r="C261" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="D261" s="17">
+      <c r="D261" s="13">
         <v>95</v>
       </c>
-      <c r="E261" s="18">
+      <c r="E261" s="14">
         <v>9.5000000000000001E-2</v>
       </c>
-      <c r="F261" s="17" t="s">
+      <c r="F261" s="13" t="s">
         <v>140</v>
       </c>
-      <c r="G261" s="18">
+      <c r="G261" s="14">
         <v>0.35799999999999998</v>
       </c>
       <c r="H261" s="2"/>
@@ -10329,19 +10543,19 @@
     </row>
     <row r="262" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A262" s="2"/>
-      <c r="B262" s="16" t="s">
+      <c r="B262" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="D262" s="19">
+      <c r="D262" s="15">
         <v>1000</v>
       </c>
-      <c r="E262" s="20">
+      <c r="E262" s="16">
         <v>1</v>
       </c>
-      <c r="F262" s="16" t="s">
+      <c r="F262" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="G262" s="20">
+      <c r="G262" s="16">
         <v>1</v>
       </c>
       <c r="H262" s="2"/>
@@ -10394,16 +10608,18 @@
     </row>
     <row r="264" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A264" s="2"/>
-      <c r="B264" s="2"/>
-      <c r="C264" s="2"/>
-      <c r="D264" s="2"/>
-      <c r="E264" s="2"/>
-      <c r="F264" s="2"/>
-      <c r="G264" s="2"/>
-      <c r="H264" s="2"/>
-      <c r="I264" s="2"/>
-      <c r="J264" s="2"/>
-      <c r="K264" s="2"/>
+      <c r="B264" s="22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C264" s="20"/>
+      <c r="D264" s="20"/>
+      <c r="E264" s="20"/>
+      <c r="F264" s="20"/>
+      <c r="G264" s="20"/>
+      <c r="H264" s="20"/>
+      <c r="I264" s="20"/>
+      <c r="J264" s="20"/>
+      <c r="K264" s="20"/>
       <c r="L264" s="2"/>
       <c r="M264" s="2"/>
       <c r="N264" s="2"/>
@@ -10422,16 +10638,36 @@
     </row>
     <row r="265" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A265" s="2"/>
-      <c r="B265" s="2"/>
-      <c r="C265" s="2"/>
-      <c r="D265" s="2"/>
-      <c r="E265" s="2"/>
-      <c r="F265" s="2"/>
-      <c r="G265" s="2"/>
-      <c r="H265" s="2"/>
-      <c r="I265" s="2"/>
-      <c r="J265" s="2"/>
-      <c r="K265" s="2"/>
+      <c r="B265" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C265" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="D265" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="E265" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="F265" s="17" t="s">
+        <v>147</v>
+      </c>
+      <c r="G265" s="17" t="s">
+        <v>148</v>
+      </c>
+      <c r="H265" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="I265" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="J265" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="K265" s="17" t="s">
+        <v>152</v>
+      </c>
       <c r="L265" s="2"/>
       <c r="M265" s="2"/>
       <c r="N265" s="2"/>
@@ -10450,16 +10686,36 @@
     </row>
     <row r="266" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A266" s="2"/>
-      <c r="B266" s="2"/>
-      <c r="C266" s="2"/>
-      <c r="D266" s="2"/>
-      <c r="E266" s="2"/>
-      <c r="F266" s="2"/>
-      <c r="G266" s="2"/>
-      <c r="H266" s="2"/>
-      <c r="I266" s="2"/>
-      <c r="J266" s="2"/>
-      <c r="K266" s="2"/>
+      <c r="B266" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C266" s="19">
+        <v>28</v>
+      </c>
+      <c r="D266" s="19">
+        <v>4</v>
+      </c>
+      <c r="E266" s="19">
+        <v>32</v>
+      </c>
+      <c r="F266" s="19">
+        <v>28</v>
+      </c>
+      <c r="G266" s="19">
+        <v>4</v>
+      </c>
+      <c r="H266" s="19">
+        <v>32</v>
+      </c>
+      <c r="I266" s="19">
+        <v>2413802</v>
+      </c>
+      <c r="J266" s="19">
+        <v>381800</v>
+      </c>
+      <c r="K266" s="19">
+        <v>2795602</v>
+      </c>
       <c r="L266" s="2"/>
       <c r="M266" s="2"/>
       <c r="N266" s="2"/>
@@ -10478,16 +10734,36 @@
     </row>
     <row r="267" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A267" s="2"/>
-      <c r="B267" s="2"/>
-      <c r="C267" s="2"/>
-      <c r="D267" s="2"/>
-      <c r="E267" s="2"/>
-      <c r="F267" s="2"/>
-      <c r="G267" s="2"/>
-      <c r="H267" s="2"/>
-      <c r="I267" s="2"/>
-      <c r="J267" s="2"/>
-      <c r="K267" s="2"/>
+      <c r="B267" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C267" s="19">
+        <v>28</v>
+      </c>
+      <c r="D267" s="19">
+        <v>2</v>
+      </c>
+      <c r="E267" s="19">
+        <v>30</v>
+      </c>
+      <c r="F267" s="19">
+        <v>28</v>
+      </c>
+      <c r="G267" s="19">
+        <v>2</v>
+      </c>
+      <c r="H267" s="19">
+        <v>30</v>
+      </c>
+      <c r="I267" s="19">
+        <v>3303124</v>
+      </c>
+      <c r="J267" s="19">
+        <v>462139</v>
+      </c>
+      <c r="K267" s="19">
+        <v>3765263</v>
+      </c>
       <c r="L267" s="2"/>
       <c r="M267" s="2"/>
       <c r="N267" s="2"/>
@@ -10506,16 +10782,36 @@
     </row>
     <row r="268" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A268" s="2"/>
-      <c r="B268" s="2"/>
-      <c r="C268" s="2"/>
-      <c r="D268" s="2"/>
-      <c r="E268" s="2"/>
-      <c r="F268" s="2"/>
-      <c r="G268" s="2"/>
-      <c r="H268" s="2"/>
-      <c r="I268" s="2"/>
-      <c r="J268" s="2"/>
-      <c r="K268" s="2"/>
+      <c r="B268" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C268" s="19">
+        <v>29</v>
+      </c>
+      <c r="D268" s="19">
+        <v>5</v>
+      </c>
+      <c r="E268" s="19">
+        <v>34</v>
+      </c>
+      <c r="F268" s="19">
+        <v>29</v>
+      </c>
+      <c r="G268" s="19">
+        <v>5</v>
+      </c>
+      <c r="H268" s="19">
+        <v>34</v>
+      </c>
+      <c r="I268" s="19">
+        <v>4169668</v>
+      </c>
+      <c r="J268" s="19">
+        <v>615917</v>
+      </c>
+      <c r="K268" s="19">
+        <v>4785585</v>
+      </c>
       <c r="L268" s="2"/>
       <c r="M268" s="2"/>
       <c r="N268" s="2"/>
@@ -10534,16 +10830,36 @@
     </row>
     <row r="269" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A269" s="2"/>
-      <c r="B269" s="2"/>
-      <c r="C269" s="2"/>
-      <c r="D269" s="2"/>
-      <c r="E269" s="2"/>
-      <c r="F269" s="2"/>
-      <c r="G269" s="2"/>
-      <c r="H269" s="2"/>
-      <c r="I269" s="2"/>
-      <c r="J269" s="2"/>
-      <c r="K269" s="2"/>
+      <c r="B269" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C269" s="19">
+        <v>12</v>
+      </c>
+      <c r="D269" s="19">
+        <v>1</v>
+      </c>
+      <c r="E269" s="19">
+        <v>13</v>
+      </c>
+      <c r="F269" s="19">
+        <v>12</v>
+      </c>
+      <c r="G269" s="19">
+        <v>1</v>
+      </c>
+      <c r="H269" s="19">
+        <v>13</v>
+      </c>
+      <c r="I269" s="19">
+        <v>1249710</v>
+      </c>
+      <c r="J269" s="19">
+        <v>106460</v>
+      </c>
+      <c r="K269" s="19">
+        <v>1356170</v>
+      </c>
       <c r="L269" s="2"/>
       <c r="M269" s="2"/>
       <c r="N269" s="2"/>
@@ -10562,16 +10878,36 @@
     </row>
     <row r="270" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A270" s="2"/>
-      <c r="B270" s="2"/>
-      <c r="C270" s="2"/>
-      <c r="D270" s="2"/>
-      <c r="E270" s="2"/>
-      <c r="F270" s="2"/>
-      <c r="G270" s="2"/>
-      <c r="H270" s="2"/>
-      <c r="I270" s="2"/>
-      <c r="J270" s="2"/>
-      <c r="K270" s="2"/>
+      <c r="B270" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C270" s="19">
+        <v>7</v>
+      </c>
+      <c r="D270" s="19">
+        <v>2</v>
+      </c>
+      <c r="E270" s="19">
+        <v>9</v>
+      </c>
+      <c r="F270" s="19">
+        <v>7</v>
+      </c>
+      <c r="G270" s="19">
+        <v>2</v>
+      </c>
+      <c r="H270" s="19">
+        <v>9</v>
+      </c>
+      <c r="I270" s="19">
+        <v>1282460</v>
+      </c>
+      <c r="J270" s="19">
+        <v>556004</v>
+      </c>
+      <c r="K270" s="19">
+        <v>1838464</v>
+      </c>
       <c r="L270" s="2"/>
       <c r="M270" s="2"/>
       <c r="N270" s="2"/>
@@ -10590,16 +10926,36 @@
     </row>
     <row r="271" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A271" s="2"/>
-      <c r="B271" s="2"/>
-      <c r="C271" s="2"/>
-      <c r="D271" s="2"/>
-      <c r="E271" s="2"/>
-      <c r="F271" s="2"/>
-      <c r="G271" s="2"/>
-      <c r="H271" s="2"/>
-      <c r="I271" s="2"/>
-      <c r="J271" s="2"/>
-      <c r="K271" s="2"/>
+      <c r="B271" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C271" s="19">
+        <v>3</v>
+      </c>
+      <c r="D271" s="19">
+        <v>1</v>
+      </c>
+      <c r="E271" s="19">
+        <v>4</v>
+      </c>
+      <c r="F271" s="19">
+        <v>3</v>
+      </c>
+      <c r="G271" s="19">
+        <v>1</v>
+      </c>
+      <c r="H271" s="19">
+        <v>4</v>
+      </c>
+      <c r="I271" s="19">
+        <v>325267</v>
+      </c>
+      <c r="J271" s="19">
+        <v>46640</v>
+      </c>
+      <c r="K271" s="19">
+        <v>371907</v>
+      </c>
       <c r="L271" s="2"/>
       <c r="M271" s="2"/>
       <c r="N271" s="2"/>
@@ -10618,16 +10974,36 @@
     </row>
     <row r="272" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A272" s="2"/>
-      <c r="B272" s="2"/>
-      <c r="C272" s="2"/>
-      <c r="D272" s="2"/>
-      <c r="E272" s="2"/>
-      <c r="F272" s="2"/>
-      <c r="G272" s="2"/>
-      <c r="H272" s="2"/>
-      <c r="I272" s="2"/>
-      <c r="J272" s="2"/>
-      <c r="K272" s="2"/>
+      <c r="B272" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C272" s="19">
+        <v>0</v>
+      </c>
+      <c r="D272" s="19">
+        <v>0</v>
+      </c>
+      <c r="E272" s="19">
+        <v>0</v>
+      </c>
+      <c r="F272" s="19">
+        <v>0</v>
+      </c>
+      <c r="G272" s="19">
+        <v>0</v>
+      </c>
+      <c r="H272" s="19">
+        <v>0</v>
+      </c>
+      <c r="I272" s="19">
+        <v>0</v>
+      </c>
+      <c r="J272" s="19">
+        <v>0</v>
+      </c>
+      <c r="K272" s="19">
+        <v>0</v>
+      </c>
       <c r="L272" s="2"/>
       <c r="M272" s="2"/>
       <c r="N272" s="2"/>
@@ -10646,16 +11022,16 @@
     </row>
     <row r="273" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A273" s="2"/>
-      <c r="B273" s="2"/>
-      <c r="C273" s="2"/>
-      <c r="D273" s="2"/>
-      <c r="E273" s="2"/>
-      <c r="F273" s="2"/>
-      <c r="G273" s="2"/>
-      <c r="H273" s="2"/>
-      <c r="I273" s="2"/>
-      <c r="J273" s="2"/>
-      <c r="K273" s="2"/>
+      <c r="B273" s="18"/>
+      <c r="C273" s="19"/>
+      <c r="D273" s="19"/>
+      <c r="E273" s="19"/>
+      <c r="F273" s="19"/>
+      <c r="G273" s="19"/>
+      <c r="H273" s="19"/>
+      <c r="I273" s="19"/>
+      <c r="J273" s="19"/>
+      <c r="K273" s="19"/>
       <c r="L273" s="2"/>
       <c r="M273" s="2"/>
       <c r="N273" s="2"/>
@@ -10674,11 +11050,13 @@
     </row>
     <row r="274" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A274" s="2"/>
-      <c r="B274" s="2"/>
-      <c r="C274" s="2"/>
-      <c r="D274" s="2"/>
-      <c r="E274" s="2"/>
-      <c r="F274" s="2"/>
+      <c r="B274" s="22" t="s">
+        <v>15</v>
+      </c>
+      <c r="C274" s="20"/>
+      <c r="D274" s="20"/>
+      <c r="E274" s="20"/>
+      <c r="F274" s="20"/>
       <c r="G274" s="2"/>
       <c r="H274" s="2"/>
       <c r="I274" s="2"/>
@@ -10702,11 +11080,21 @@
     </row>
     <row r="275" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A275" s="2"/>
-      <c r="B275" s="2"/>
-      <c r="C275" s="2"/>
-      <c r="D275" s="2"/>
-      <c r="E275" s="2"/>
-      <c r="F275" s="2"/>
+      <c r="B275" s="17" t="s">
+        <v>154</v>
+      </c>
+      <c r="C275" s="17" t="s">
+        <v>155</v>
+      </c>
+      <c r="D275" s="17" t="s">
+        <v>156</v>
+      </c>
+      <c r="E275" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="F275" s="17" t="s">
+        <v>158</v>
+      </c>
       <c r="G275" s="2"/>
       <c r="H275" s="2"/>
       <c r="I275" s="2"/>
@@ -10730,11 +11118,21 @@
     </row>
     <row r="276" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A276" s="2"/>
-      <c r="B276" s="2"/>
-      <c r="C276" s="2"/>
-      <c r="D276" s="2"/>
-      <c r="E276" s="2"/>
-      <c r="F276" s="2"/>
+      <c r="B276" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="C276" s="19">
+        <v>9</v>
+      </c>
+      <c r="D276" s="19">
+        <v>22.5</v>
+      </c>
+      <c r="E276" s="19">
+        <v>3749246</v>
+      </c>
+      <c r="F276" s="19">
+        <v>50.31</v>
+      </c>
       <c r="G276" s="2"/>
       <c r="H276" s="2"/>
       <c r="I276" s="2"/>
@@ -10758,11 +11156,21 @@
     </row>
     <row r="277" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A277" s="2"/>
-      <c r="B277" s="2"/>
-      <c r="C277" s="2"/>
-      <c r="D277" s="2"/>
-      <c r="E277" s="2"/>
-      <c r="F277" s="2"/>
+      <c r="B277" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="C277" s="19">
+        <v>7</v>
+      </c>
+      <c r="D277" s="19">
+        <v>17.5</v>
+      </c>
+      <c r="E277" s="19">
+        <v>1000619</v>
+      </c>
+      <c r="F277" s="19">
+        <v>13.43</v>
+      </c>
       <c r="G277" s="2"/>
       <c r="H277" s="2"/>
       <c r="I277" s="2"/>
@@ -10786,11 +11194,21 @@
     </row>
     <row r="278" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A278" s="2"/>
-      <c r="B278" s="2"/>
-      <c r="C278" s="2"/>
-      <c r="D278" s="2"/>
-      <c r="E278" s="2"/>
-      <c r="F278" s="2"/>
+      <c r="B278" s="17" t="s">
+        <v>56</v>
+      </c>
+      <c r="C278" s="19">
+        <v>6</v>
+      </c>
+      <c r="D278" s="19">
+        <v>15</v>
+      </c>
+      <c r="E278" s="19">
+        <v>649164</v>
+      </c>
+      <c r="F278" s="19">
+        <v>8.7100000000000009</v>
+      </c>
       <c r="G278" s="2"/>
       <c r="H278" s="2"/>
       <c r="I278" s="2"/>
@@ -10814,11 +11232,21 @@
     </row>
     <row r="279" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A279" s="2"/>
-      <c r="B279" s="2"/>
-      <c r="C279" s="2"/>
-      <c r="D279" s="2"/>
-      <c r="E279" s="2"/>
-      <c r="F279" s="2"/>
+      <c r="B279" s="17" t="s">
+        <v>59</v>
+      </c>
+      <c r="C279" s="19">
+        <v>6</v>
+      </c>
+      <c r="D279" s="19">
+        <v>15</v>
+      </c>
+      <c r="E279" s="19">
+        <v>586993</v>
+      </c>
+      <c r="F279" s="19">
+        <v>7.88</v>
+      </c>
       <c r="G279" s="2"/>
       <c r="H279" s="2"/>
       <c r="I279" s="2"/>
@@ -10842,11 +11270,21 @@
     </row>
     <row r="280" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A280" s="2"/>
-      <c r="B280" s="2"/>
-      <c r="C280" s="2"/>
-      <c r="D280" s="2"/>
-      <c r="E280" s="2"/>
-      <c r="F280" s="2"/>
+      <c r="B280" s="17" t="s">
+        <v>57</v>
+      </c>
+      <c r="C280" s="19">
+        <v>3</v>
+      </c>
+      <c r="D280" s="19">
+        <v>7.5</v>
+      </c>
+      <c r="E280" s="19">
+        <v>455923</v>
+      </c>
+      <c r="F280" s="19">
+        <v>6.12</v>
+      </c>
       <c r="G280" s="2"/>
       <c r="H280" s="2"/>
       <c r="I280" s="2"/>
@@ -10870,11 +11308,21 @@
     </row>
     <row r="281" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A281" s="2"/>
-      <c r="B281" s="2"/>
-      <c r="C281" s="2"/>
-      <c r="D281" s="2"/>
-      <c r="E281" s="2"/>
-      <c r="F281" s="2"/>
+      <c r="B281" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="C281" s="19">
+        <v>4</v>
+      </c>
+      <c r="D281" s="19">
+        <v>10</v>
+      </c>
+      <c r="E281" s="19">
+        <v>378219</v>
+      </c>
+      <c r="F281" s="19">
+        <v>5.08</v>
+      </c>
       <c r="G281" s="2"/>
       <c r="H281" s="2"/>
       <c r="I281" s="2"/>
@@ -10898,11 +11346,21 @@
     </row>
     <row r="282" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A282" s="2"/>
-      <c r="B282" s="2"/>
-      <c r="C282" s="2"/>
-      <c r="D282" s="2"/>
-      <c r="E282" s="2"/>
-      <c r="F282" s="2"/>
+      <c r="B282" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="C282" s="19">
+        <v>2</v>
+      </c>
+      <c r="D282" s="19">
+        <v>5</v>
+      </c>
+      <c r="E282" s="19">
+        <v>233510</v>
+      </c>
+      <c r="F282" s="19">
+        <v>3.13</v>
+      </c>
       <c r="G282" s="2"/>
       <c r="H282" s="2"/>
       <c r="I282" s="2"/>
@@ -10926,11 +11384,21 @@
     </row>
     <row r="283" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A283" s="2"/>
-      <c r="B283" s="2"/>
-      <c r="C283" s="2"/>
-      <c r="D283" s="2"/>
-      <c r="E283" s="2"/>
-      <c r="F283" s="2"/>
+      <c r="B283" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="C283" s="19">
+        <v>2</v>
+      </c>
+      <c r="D283" s="19">
+        <v>5</v>
+      </c>
+      <c r="E283" s="19">
+        <v>227982</v>
+      </c>
+      <c r="F283" s="19">
+        <v>3.06</v>
+      </c>
       <c r="G283" s="2"/>
       <c r="H283" s="2"/>
       <c r="I283" s="2"/>
@@ -10954,11 +11422,21 @@
     </row>
     <row r="284" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A284" s="2"/>
-      <c r="B284" s="2"/>
-      <c r="C284" s="2"/>
-      <c r="D284" s="2"/>
-      <c r="E284" s="2"/>
-      <c r="F284" s="2"/>
+      <c r="B284" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="C284" s="19">
+        <v>1</v>
+      </c>
+      <c r="D284" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="E284" s="19">
+        <v>170320</v>
+      </c>
+      <c r="F284" s="19">
+        <v>2.29</v>
+      </c>
       <c r="G284" s="2"/>
       <c r="H284" s="2"/>
       <c r="I284" s="2"/>
@@ -11010,16 +11488,6 @@
     </row>
     <row r="286" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A286" s="2"/>
-      <c r="B286" s="2"/>
-      <c r="C286" s="2"/>
-      <c r="D286" s="2"/>
-      <c r="E286" s="2"/>
-      <c r="F286" s="2"/>
-      <c r="G286" s="2"/>
-      <c r="H286" s="2"/>
-      <c r="I286" s="2"/>
-      <c r="J286" s="2"/>
-      <c r="K286" s="2"/>
       <c r="L286" s="2"/>
       <c r="M286" s="2"/>
       <c r="N286" s="2"/>
@@ -11038,16 +11506,18 @@
     </row>
     <row r="287" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A287" s="2"/>
-      <c r="B287" s="2"/>
-      <c r="C287" s="2"/>
-      <c r="D287" s="2"/>
-      <c r="E287" s="2"/>
-      <c r="F287" s="2"/>
-      <c r="G287" s="2"/>
-      <c r="H287" s="2"/>
-      <c r="I287" s="2"/>
-      <c r="J287" s="2"/>
-      <c r="K287" s="2"/>
+      <c r="B287" s="22" t="s">
+        <v>166</v>
+      </c>
+      <c r="C287" s="20"/>
+      <c r="D287" s="20"/>
+      <c r="E287" s="20"/>
+      <c r="F287" s="20"/>
+      <c r="G287" s="20"/>
+      <c r="H287" s="20"/>
+      <c r="I287" s="20"/>
+      <c r="J287" s="20"/>
+      <c r="K287" s="20"/>
       <c r="L287" s="2"/>
       <c r="M287" s="2"/>
       <c r="N287" s="2"/>
@@ -11066,16 +11536,36 @@
     </row>
     <row r="288" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A288" s="2"/>
-      <c r="B288" s="2"/>
-      <c r="C288" s="2"/>
-      <c r="D288" s="2"/>
-      <c r="E288" s="2"/>
-      <c r="F288" s="2"/>
-      <c r="G288" s="2"/>
-      <c r="H288" s="2"/>
-      <c r="I288" s="2"/>
-      <c r="J288" s="2"/>
-      <c r="K288" s="2"/>
+      <c r="B288" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="C288" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="D288" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="E288" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="F288" s="17" t="s">
+        <v>149</v>
+      </c>
+      <c r="G288" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="H288" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="I288" s="17" t="s">
+        <v>162</v>
+      </c>
+      <c r="J288" s="17" t="s">
+        <v>163</v>
+      </c>
+      <c r="K288" s="17" t="s">
+        <v>164</v>
+      </c>
       <c r="L288" s="2"/>
       <c r="M288" s="2"/>
       <c r="N288" s="2"/>
@@ -11094,16 +11584,36 @@
     </row>
     <row r="289" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A289" s="2"/>
-      <c r="B289" s="2"/>
-      <c r="C289" s="2"/>
-      <c r="D289" s="2"/>
-      <c r="E289" s="2"/>
-      <c r="F289" s="2"/>
-      <c r="G289" s="2"/>
-      <c r="H289" s="2"/>
-      <c r="I289" s="2"/>
-      <c r="J289" s="2"/>
-      <c r="K289" s="2"/>
+      <c r="B289" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C289" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D289" s="19">
+        <v>26</v>
+      </c>
+      <c r="E289" s="19">
+        <v>11.11</v>
+      </c>
+      <c r="F289" s="19">
+        <v>28</v>
+      </c>
+      <c r="G289" s="19">
+        <v>3748727</v>
+      </c>
+      <c r="H289" s="19">
+        <v>13.84</v>
+      </c>
+      <c r="I289" s="19">
+        <v>1.04</v>
+      </c>
+      <c r="J289" s="19">
+        <v>1.42</v>
+      </c>
+      <c r="K289" s="19">
+        <v>180594.85</v>
+      </c>
       <c r="L289" s="2"/>
       <c r="M289" s="2"/>
       <c r="N289" s="2"/>
@@ -11122,16 +11632,36 @@
     </row>
     <row r="290" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A290" s="2"/>
-      <c r="B290" s="2"/>
-      <c r="C290" s="2"/>
-      <c r="D290" s="2"/>
-      <c r="E290" s="2"/>
-      <c r="F290" s="2"/>
-      <c r="G290" s="2"/>
-      <c r="H290" s="2"/>
-      <c r="I290" s="2"/>
-      <c r="J290" s="2"/>
-      <c r="K290" s="2"/>
+      <c r="B290" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C290" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D290" s="19">
+        <v>29</v>
+      </c>
+      <c r="E290" s="19">
+        <v>12.39</v>
+      </c>
+      <c r="F290" s="19">
+        <v>29</v>
+      </c>
+      <c r="G290" s="19">
+        <v>6953013</v>
+      </c>
+      <c r="H290" s="19">
+        <v>25.67</v>
+      </c>
+      <c r="I290" s="19">
+        <v>2</v>
+      </c>
+      <c r="J290" s="19">
+        <v>1.24</v>
+      </c>
+      <c r="K290" s="19">
+        <v>258966.93</v>
+      </c>
       <c r="L290" s="2"/>
       <c r="M290" s="2"/>
       <c r="N290" s="2"/>
@@ -11150,16 +11680,36 @@
     </row>
     <row r="291" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A291" s="2"/>
-      <c r="B291" s="2"/>
-      <c r="C291" s="2"/>
-      <c r="D291" s="2"/>
-      <c r="E291" s="2"/>
-      <c r="F291" s="2"/>
-      <c r="G291" s="2"/>
-      <c r="H291" s="2"/>
-      <c r="I291" s="2"/>
-      <c r="J291" s="2"/>
-      <c r="K291" s="2"/>
+      <c r="B291" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C291" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D291" s="19">
+        <v>56</v>
+      </c>
+      <c r="E291" s="19">
+        <v>23.93</v>
+      </c>
+      <c r="F291" s="19">
+        <v>57</v>
+      </c>
+      <c r="G291" s="19">
+        <v>3588440</v>
+      </c>
+      <c r="H291" s="19">
+        <v>13.25</v>
+      </c>
+      <c r="I291" s="19">
+        <v>0.77</v>
+      </c>
+      <c r="J291" s="19">
+        <v>1.02</v>
+      </c>
+      <c r="K291" s="19">
+        <v>64079.29</v>
+      </c>
       <c r="L291" s="2"/>
       <c r="M291" s="2"/>
       <c r="N291" s="2"/>
@@ -11178,16 +11728,36 @@
     </row>
     <row r="292" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A292" s="2"/>
-      <c r="B292" s="2"/>
-      <c r="C292" s="2"/>
-      <c r="D292" s="2"/>
-      <c r="E292" s="2"/>
-      <c r="F292" s="2"/>
-      <c r="G292" s="2"/>
-      <c r="H292" s="2"/>
-      <c r="I292" s="2"/>
-      <c r="J292" s="2"/>
-      <c r="K292" s="2"/>
+      <c r="B292" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C292" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D292" s="19">
+        <v>123</v>
+      </c>
+      <c r="E292" s="19">
+        <v>52.56</v>
+      </c>
+      <c r="F292" s="19">
+        <v>123</v>
+      </c>
+      <c r="G292" s="19">
+        <v>12793257</v>
+      </c>
+      <c r="H292" s="19">
+        <v>47.24</v>
+      </c>
+      <c r="I292" s="19">
+        <v>4.37</v>
+      </c>
+      <c r="J292" s="19">
+        <v>1.24</v>
+      </c>
+      <c r="K292" s="19">
+        <v>137730.28</v>
+      </c>
       <c r="L292" s="2"/>
       <c r="M292" s="2"/>
       <c r="N292" s="2"/>
@@ -11206,16 +11776,36 @@
     </row>
     <row r="293" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A293" s="2"/>
-      <c r="B293" s="2"/>
-      <c r="C293" s="2"/>
-      <c r="D293" s="2"/>
-      <c r="E293" s="2"/>
-      <c r="F293" s="2"/>
-      <c r="G293" s="2"/>
-      <c r="H293" s="2"/>
-      <c r="I293" s="2"/>
-      <c r="J293" s="2"/>
-      <c r="K293" s="2"/>
+      <c r="B293" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C293" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D293" s="19">
+        <v>28</v>
+      </c>
+      <c r="E293" s="19">
+        <v>11.86</v>
+      </c>
+      <c r="F293" s="19">
+        <v>30</v>
+      </c>
+      <c r="G293" s="19">
+        <v>4313780</v>
+      </c>
+      <c r="H293" s="19">
+        <v>16.22</v>
+      </c>
+      <c r="I293" s="19">
+        <v>0.96</v>
+      </c>
+      <c r="J293" s="19">
+        <v>1.25</v>
+      </c>
+      <c r="K293" s="19">
+        <v>177533.54</v>
+      </c>
       <c r="L293" s="2"/>
       <c r="M293" s="2"/>
       <c r="N293" s="2"/>
@@ -11234,16 +11824,36 @@
     </row>
     <row r="294" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A294" s="2"/>
-      <c r="B294" s="2"/>
-      <c r="C294" s="2"/>
-      <c r="D294" s="2"/>
-      <c r="E294" s="2"/>
-      <c r="F294" s="2"/>
-      <c r="G294" s="2"/>
-      <c r="H294" s="2"/>
-      <c r="I294" s="2"/>
-      <c r="J294" s="2"/>
-      <c r="K294" s="2"/>
+      <c r="B294" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C294" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D294" s="19">
+        <v>34</v>
+      </c>
+      <c r="E294" s="19">
+        <v>14.41</v>
+      </c>
+      <c r="F294" s="19">
+        <v>34</v>
+      </c>
+      <c r="G294" s="19">
+        <v>7209305</v>
+      </c>
+      <c r="H294" s="19">
+        <v>27.11</v>
+      </c>
+      <c r="I294" s="19">
+        <v>2.38</v>
+      </c>
+      <c r="J294" s="19">
+        <v>1.35</v>
+      </c>
+      <c r="K294" s="19">
+        <v>244556.26</v>
+      </c>
       <c r="L294" s="2"/>
       <c r="M294" s="2"/>
       <c r="N294" s="2"/>
@@ -11262,16 +11872,36 @@
     </row>
     <row r="295" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A295" s="2"/>
-      <c r="B295" s="2"/>
-      <c r="C295" s="2"/>
-      <c r="D295" s="2"/>
-      <c r="E295" s="2"/>
-      <c r="F295" s="2"/>
-      <c r="G295" s="2"/>
-      <c r="H295" s="2"/>
-      <c r="I295" s="2"/>
-      <c r="J295" s="2"/>
-      <c r="K295" s="2"/>
+      <c r="B295" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C295" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D295" s="19">
+        <v>58</v>
+      </c>
+      <c r="E295" s="19">
+        <v>24.58</v>
+      </c>
+      <c r="F295" s="19">
+        <v>59</v>
+      </c>
+      <c r="G295" s="19">
+        <v>3724296</v>
+      </c>
+      <c r="H295" s="19">
+        <v>14</v>
+      </c>
+      <c r="I295" s="19">
+        <v>1.05</v>
+      </c>
+      <c r="J295" s="19">
+        <v>1.02</v>
+      </c>
+      <c r="K295" s="19">
+        <v>64212</v>
+      </c>
       <c r="L295" s="2"/>
       <c r="M295" s="2"/>
       <c r="N295" s="2"/>
@@ -11290,16 +11920,36 @@
     </row>
     <row r="296" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A296" s="2"/>
-      <c r="B296" s="2"/>
-      <c r="C296" s="2"/>
-      <c r="D296" s="2"/>
-      <c r="E296" s="2"/>
-      <c r="F296" s="2"/>
-      <c r="G296" s="2"/>
-      <c r="H296" s="2"/>
-      <c r="I296" s="2"/>
-      <c r="J296" s="2"/>
-      <c r="K296" s="2"/>
+      <c r="B296" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C296" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D296" s="19">
+        <v>116</v>
+      </c>
+      <c r="E296" s="19">
+        <v>49.15</v>
+      </c>
+      <c r="F296" s="19">
+        <v>116</v>
+      </c>
+      <c r="G296" s="19">
+        <v>11350179</v>
+      </c>
+      <c r="H296" s="19">
+        <v>42.67</v>
+      </c>
+      <c r="I296" s="19">
+        <v>4.6100000000000003</v>
+      </c>
+      <c r="J296" s="19">
+        <v>1.17</v>
+      </c>
+      <c r="K296" s="19">
+        <v>122884.03</v>
+      </c>
       <c r="L296" s="2"/>
       <c r="M296" s="2"/>
       <c r="N296" s="2"/>
@@ -11318,16 +11968,36 @@
     </row>
     <row r="297" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A297" s="2"/>
-      <c r="B297" s="2"/>
-      <c r="C297" s="2"/>
-      <c r="D297" s="2"/>
-      <c r="E297" s="2"/>
-      <c r="F297" s="2"/>
-      <c r="G297" s="2"/>
-      <c r="H297" s="2"/>
-      <c r="I297" s="2"/>
-      <c r="J297" s="2"/>
-      <c r="K297" s="2"/>
+      <c r="B297" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C297" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D297" s="19">
+        <v>25</v>
+      </c>
+      <c r="E297" s="19">
+        <v>10.46</v>
+      </c>
+      <c r="F297" s="19">
+        <v>27</v>
+      </c>
+      <c r="G297" s="19">
+        <v>3833837</v>
+      </c>
+      <c r="H297" s="19">
+        <v>13.33</v>
+      </c>
+      <c r="I297" s="19">
+        <v>0.88</v>
+      </c>
+      <c r="J297" s="19">
+        <v>1.28</v>
+      </c>
+      <c r="K297" s="19">
+        <v>177890.44</v>
+      </c>
       <c r="L297" s="2"/>
       <c r="M297" s="2"/>
       <c r="N297" s="2"/>
@@ -11346,16 +12016,36 @@
     </row>
     <row r="298" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A298" s="2"/>
-      <c r="B298" s="2"/>
-      <c r="C298" s="2"/>
-      <c r="D298" s="2"/>
-      <c r="E298" s="2"/>
-      <c r="F298" s="2"/>
-      <c r="G298" s="2"/>
-      <c r="H298" s="2"/>
-      <c r="I298" s="2"/>
-      <c r="J298" s="2"/>
-      <c r="K298" s="2"/>
+      <c r="B298" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C298" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D298" s="19">
+        <v>29</v>
+      </c>
+      <c r="E298" s="19">
+        <v>12.13</v>
+      </c>
+      <c r="F298" s="19">
+        <v>29</v>
+      </c>
+      <c r="G298" s="19">
+        <v>7122117</v>
+      </c>
+      <c r="H298" s="19">
+        <v>24.76</v>
+      </c>
+      <c r="I298" s="19">
+        <v>2.14</v>
+      </c>
+      <c r="J298" s="19">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K298" s="19">
+        <v>257616.72</v>
+      </c>
       <c r="L298" s="2"/>
       <c r="M298" s="2"/>
       <c r="N298" s="2"/>
@@ -11374,16 +12064,36 @@
     </row>
     <row r="299" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A299" s="2"/>
-      <c r="B299" s="2"/>
-      <c r="C299" s="2"/>
-      <c r="D299" s="2"/>
-      <c r="E299" s="2"/>
-      <c r="F299" s="2"/>
-      <c r="G299" s="2"/>
-      <c r="H299" s="2"/>
-      <c r="I299" s="2"/>
-      <c r="J299" s="2"/>
-      <c r="K299" s="2"/>
+      <c r="B299" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C299" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D299" s="19">
+        <v>60</v>
+      </c>
+      <c r="E299" s="19">
+        <v>25.1</v>
+      </c>
+      <c r="F299" s="19">
+        <v>61</v>
+      </c>
+      <c r="G299" s="19">
+        <v>3792882</v>
+      </c>
+      <c r="H299" s="19">
+        <v>13.18</v>
+      </c>
+      <c r="I299" s="19">
+        <v>1.08</v>
+      </c>
+      <c r="J299" s="19">
+        <v>1.05</v>
+      </c>
+      <c r="K299" s="19">
+        <v>63986.65</v>
+      </c>
       <c r="L299" s="2"/>
       <c r="M299" s="2"/>
       <c r="N299" s="2"/>
@@ -11402,16 +12112,36 @@
     </row>
     <row r="300" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A300" s="2"/>
-      <c r="B300" s="2"/>
-      <c r="C300" s="2"/>
-      <c r="D300" s="2"/>
-      <c r="E300" s="2"/>
-      <c r="F300" s="2"/>
-      <c r="G300" s="2"/>
-      <c r="H300" s="2"/>
-      <c r="I300" s="2"/>
-      <c r="J300" s="2"/>
-      <c r="K300" s="2"/>
+      <c r="B300" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C300" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D300" s="19">
+        <v>125</v>
+      </c>
+      <c r="E300" s="19">
+        <v>52.3</v>
+      </c>
+      <c r="F300" s="19">
+        <v>125</v>
+      </c>
+      <c r="G300" s="19">
+        <v>14019341</v>
+      </c>
+      <c r="H300" s="19">
+        <v>48.73</v>
+      </c>
+      <c r="I300" s="19">
+        <v>4.59</v>
+      </c>
+      <c r="J300" s="19">
+        <v>1.18</v>
+      </c>
+      <c r="K300" s="19">
+        <v>134885.6</v>
+      </c>
       <c r="L300" s="2"/>
       <c r="M300" s="2"/>
       <c r="N300" s="2"/>
@@ -11430,16 +12160,36 @@
     </row>
     <row r="301" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A301" s="2"/>
-      <c r="B301" s="2"/>
-      <c r="C301" s="2"/>
-      <c r="D301" s="2"/>
-      <c r="E301" s="2"/>
-      <c r="F301" s="2"/>
-      <c r="G301" s="2"/>
-      <c r="H301" s="2"/>
-      <c r="I301" s="2"/>
-      <c r="J301" s="2"/>
-      <c r="K301" s="2"/>
+      <c r="B301" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C301" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D301" s="19">
+        <v>22</v>
+      </c>
+      <c r="E301" s="19">
+        <v>9.9499999999999993</v>
+      </c>
+      <c r="F301" s="19">
+        <v>22</v>
+      </c>
+      <c r="G301" s="19">
+        <v>3443999</v>
+      </c>
+      <c r="H301" s="19">
+        <v>12.8</v>
+      </c>
+      <c r="I301" s="19">
+        <v>1.36</v>
+      </c>
+      <c r="J301" s="19">
+        <v>1.18</v>
+      </c>
+      <c r="K301" s="19">
+        <v>179934.73</v>
+      </c>
       <c r="L301" s="2"/>
       <c r="M301" s="2"/>
       <c r="N301" s="2"/>
@@ -11458,16 +12208,36 @@
     </row>
     <row r="302" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A302" s="2"/>
-      <c r="B302" s="2"/>
-      <c r="C302" s="2"/>
-      <c r="D302" s="2"/>
-      <c r="E302" s="2"/>
-      <c r="F302" s="2"/>
-      <c r="G302" s="2"/>
-      <c r="H302" s="2"/>
-      <c r="I302" s="2"/>
-      <c r="J302" s="2"/>
-      <c r="K302" s="2"/>
+      <c r="B302" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C302" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D302" s="19">
+        <v>29</v>
+      </c>
+      <c r="E302" s="19">
+        <v>13.12</v>
+      </c>
+      <c r="F302" s="19">
+        <v>31</v>
+      </c>
+      <c r="G302" s="19">
+        <v>7106763</v>
+      </c>
+      <c r="H302" s="19">
+        <v>26.42</v>
+      </c>
+      <c r="I302" s="19">
+        <v>2.86</v>
+      </c>
+      <c r="J302" s="19">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="K302" s="19">
+        <v>251721.45</v>
+      </c>
       <c r="L302" s="2"/>
       <c r="M302" s="2"/>
       <c r="N302" s="2"/>
@@ -11486,16 +12256,36 @@
     </row>
     <row r="303" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A303" s="2"/>
-      <c r="B303" s="2"/>
-      <c r="C303" s="2"/>
-      <c r="D303" s="2"/>
-      <c r="E303" s="2"/>
-      <c r="F303" s="2"/>
-      <c r="G303" s="2"/>
-      <c r="H303" s="2"/>
-      <c r="I303" s="2"/>
-      <c r="J303" s="2"/>
-      <c r="K303" s="2"/>
+      <c r="B303" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C303" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D303" s="19">
+        <v>58</v>
+      </c>
+      <c r="E303" s="19">
+        <v>26.24</v>
+      </c>
+      <c r="F303" s="19">
+        <v>58</v>
+      </c>
+      <c r="G303" s="19">
+        <v>3570376</v>
+      </c>
+      <c r="H303" s="19">
+        <v>13.27</v>
+      </c>
+      <c r="I303" s="19">
+        <v>1.53</v>
+      </c>
+      <c r="J303" s="19">
+        <v>1.03</v>
+      </c>
+      <c r="K303" s="19">
+        <v>62356.78</v>
+      </c>
       <c r="L303" s="2"/>
       <c r="M303" s="2"/>
       <c r="N303" s="2"/>
@@ -11514,16 +12304,36 @@
     </row>
     <row r="304" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A304" s="2"/>
-      <c r="B304" s="2"/>
-      <c r="C304" s="2"/>
-      <c r="D304" s="2"/>
-      <c r="E304" s="2"/>
-      <c r="F304" s="2"/>
-      <c r="G304" s="2"/>
-      <c r="H304" s="2"/>
-      <c r="I304" s="2"/>
-      <c r="J304" s="2"/>
-      <c r="K304" s="2"/>
+      <c r="B304" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C304" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D304" s="19">
+        <v>112</v>
+      </c>
+      <c r="E304" s="19">
+        <v>50.68</v>
+      </c>
+      <c r="F304" s="19">
+        <v>112</v>
+      </c>
+      <c r="G304" s="19">
+        <v>12781586</v>
+      </c>
+      <c r="H304" s="19">
+        <v>47.51</v>
+      </c>
+      <c r="I304" s="19">
+        <v>4.8499999999999996</v>
+      </c>
+      <c r="J304" s="19">
+        <v>1.19</v>
+      </c>
+      <c r="K304" s="19">
+        <v>137551.38</v>
+      </c>
       <c r="L304" s="2"/>
       <c r="M304" s="2"/>
       <c r="N304" s="2"/>
@@ -11542,16 +12352,36 @@
     </row>
     <row r="305" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A305" s="2"/>
-      <c r="B305" s="2"/>
-      <c r="C305" s="2"/>
-      <c r="D305" s="2"/>
-      <c r="E305" s="2"/>
-      <c r="F305" s="2"/>
-      <c r="G305" s="2"/>
-      <c r="H305" s="2"/>
-      <c r="I305" s="2"/>
-      <c r="J305" s="2"/>
-      <c r="K305" s="2"/>
+      <c r="B305" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C305" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D305" s="19">
+        <v>19</v>
+      </c>
+      <c r="E305" s="19">
+        <v>9.69</v>
+      </c>
+      <c r="F305" s="19">
+        <v>19</v>
+      </c>
+      <c r="G305" s="19">
+        <v>3302523</v>
+      </c>
+      <c r="H305" s="19">
+        <v>13.41</v>
+      </c>
+      <c r="I305" s="19">
+        <v>1.58</v>
+      </c>
+      <c r="J305" s="19">
+        <v>1.1599999999999999</v>
+      </c>
+      <c r="K305" s="19">
+        <v>198558.32</v>
+      </c>
       <c r="L305" s="2"/>
       <c r="M305" s="2"/>
       <c r="N305" s="2"/>
@@ -11570,16 +12400,36 @@
     </row>
     <row r="306" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A306" s="2"/>
-      <c r="B306" s="2"/>
-      <c r="C306" s="2"/>
-      <c r="D306" s="2"/>
-      <c r="E306" s="2"/>
-      <c r="F306" s="2"/>
-      <c r="G306" s="2"/>
-      <c r="H306" s="2"/>
-      <c r="I306" s="2"/>
-      <c r="J306" s="2"/>
-      <c r="K306" s="2"/>
+      <c r="B306" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C306" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D306" s="19">
+        <v>23</v>
+      </c>
+      <c r="E306" s="19">
+        <v>11.73</v>
+      </c>
+      <c r="F306" s="19">
+        <v>25</v>
+      </c>
+      <c r="G306" s="19">
+        <v>5533319</v>
+      </c>
+      <c r="H306" s="19">
+        <v>22.46</v>
+      </c>
+      <c r="I306" s="19">
+        <v>2.96</v>
+      </c>
+      <c r="J306" s="19">
+        <v>1.22</v>
+      </c>
+      <c r="K306" s="19">
+        <v>259833.83</v>
+      </c>
       <c r="L306" s="2"/>
       <c r="M306" s="2"/>
       <c r="N306" s="2"/>
@@ -11598,16 +12448,36 @@
     </row>
     <row r="307" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A307" s="2"/>
-      <c r="B307" s="2"/>
-      <c r="C307" s="2"/>
-      <c r="D307" s="2"/>
-      <c r="E307" s="2"/>
-      <c r="F307" s="2"/>
-      <c r="G307" s="2"/>
-      <c r="H307" s="2"/>
-      <c r="I307" s="2"/>
-      <c r="J307" s="2"/>
-      <c r="K307" s="2"/>
+      <c r="B307" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C307" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D307" s="19">
+        <v>52</v>
+      </c>
+      <c r="E307" s="19">
+        <v>26.53</v>
+      </c>
+      <c r="F307" s="19">
+        <v>52</v>
+      </c>
+      <c r="G307" s="19">
+        <v>4449851</v>
+      </c>
+      <c r="H307" s="19">
+        <v>18.059999999999999</v>
+      </c>
+      <c r="I307" s="19">
+        <v>2.02</v>
+      </c>
+      <c r="J307" s="19">
+        <v>1.04</v>
+      </c>
+      <c r="K307" s="19">
+        <v>86464.77</v>
+      </c>
       <c r="L307" s="2"/>
       <c r="M307" s="2"/>
       <c r="N307" s="2"/>
@@ -11626,16 +12496,36 @@
     </row>
     <row r="308" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A308" s="2"/>
-      <c r="B308" s="2"/>
-      <c r="C308" s="2"/>
-      <c r="D308" s="2"/>
-      <c r="E308" s="2"/>
-      <c r="F308" s="2"/>
-      <c r="G308" s="2"/>
-      <c r="H308" s="2"/>
-      <c r="I308" s="2"/>
-      <c r="J308" s="2"/>
-      <c r="K308" s="2"/>
+      <c r="B308" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C308" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D308" s="19">
+        <v>102</v>
+      </c>
+      <c r="E308" s="19">
+        <v>52.04</v>
+      </c>
+      <c r="F308" s="19">
+        <v>102</v>
+      </c>
+      <c r="G308" s="19">
+        <v>11347882</v>
+      </c>
+      <c r="H308" s="19">
+        <v>46.07</v>
+      </c>
+      <c r="I308" s="19">
+        <v>5.15</v>
+      </c>
+      <c r="J308" s="19">
+        <v>1.1499999999999999</v>
+      </c>
+      <c r="K308" s="19">
+        <v>124458.73</v>
+      </c>
       <c r="L308" s="2"/>
       <c r="M308" s="2"/>
       <c r="N308" s="2"/>
@@ -11654,16 +12544,36 @@
     </row>
     <row r="309" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A309" s="2"/>
-      <c r="B309" s="2"/>
-      <c r="C309" s="2"/>
-      <c r="D309" s="2"/>
-      <c r="E309" s="2"/>
-      <c r="F309" s="2"/>
-      <c r="G309" s="2"/>
-      <c r="H309" s="2"/>
-      <c r="I309" s="2"/>
-      <c r="J309" s="2"/>
-      <c r="K309" s="2"/>
+      <c r="B309" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C309" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D309" s="19">
+        <v>18</v>
+      </c>
+      <c r="E309" s="19">
+        <v>11.18</v>
+      </c>
+      <c r="F309" s="19">
+        <v>18</v>
+      </c>
+      <c r="G309" s="19">
+        <v>3123684</v>
+      </c>
+      <c r="H309" s="19">
+        <v>15.83</v>
+      </c>
+      <c r="I309" s="19">
+        <v>2.17</v>
+      </c>
+      <c r="J309" s="19">
+        <v>1.17</v>
+      </c>
+      <c r="K309" s="19">
+        <v>199653.83</v>
+      </c>
       <c r="L309" s="2"/>
       <c r="M309" s="2"/>
       <c r="N309" s="2"/>
@@ -11682,16 +12592,36 @@
     </row>
     <row r="310" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A310" s="2"/>
-      <c r="B310" s="2"/>
-      <c r="C310" s="2"/>
-      <c r="D310" s="2"/>
-      <c r="E310" s="2"/>
-      <c r="F310" s="2"/>
-      <c r="G310" s="2"/>
-      <c r="H310" s="2"/>
-      <c r="I310" s="2"/>
-      <c r="J310" s="2"/>
-      <c r="K310" s="2"/>
+      <c r="B310" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C310" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D310" s="19">
+        <v>19</v>
+      </c>
+      <c r="E310" s="19">
+        <v>11.8</v>
+      </c>
+      <c r="F310" s="19">
+        <v>19</v>
+      </c>
+      <c r="G310" s="19">
+        <v>4562138</v>
+      </c>
+      <c r="H310" s="19">
+        <v>23.12</v>
+      </c>
+      <c r="I310" s="19">
+        <v>3.53</v>
+      </c>
+      <c r="J310" s="19">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="K310" s="19">
+        <v>258217.79</v>
+      </c>
       <c r="L310" s="2"/>
       <c r="M310" s="2"/>
       <c r="N310" s="2"/>
@@ -11710,16 +12640,36 @@
     </row>
     <row r="311" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A311" s="2"/>
-      <c r="B311" s="2"/>
-      <c r="C311" s="2"/>
-      <c r="D311" s="2"/>
-      <c r="E311" s="2"/>
-      <c r="F311" s="2"/>
-      <c r="G311" s="2"/>
-      <c r="H311" s="2"/>
-      <c r="I311" s="2"/>
-      <c r="J311" s="2"/>
-      <c r="K311" s="2"/>
+      <c r="B311" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C311" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D311" s="19">
+        <v>41</v>
+      </c>
+      <c r="E311" s="19">
+        <v>25.47</v>
+      </c>
+      <c r="F311" s="19">
+        <v>41</v>
+      </c>
+      <c r="G311" s="19">
+        <v>3408463</v>
+      </c>
+      <c r="H311" s="19">
+        <v>17.28</v>
+      </c>
+      <c r="I311" s="19">
+        <v>2.5099999999999998</v>
+      </c>
+      <c r="J311" s="19">
+        <v>1.05</v>
+      </c>
+      <c r="K311" s="19">
+        <v>84262.93</v>
+      </c>
       <c r="L311" s="2"/>
       <c r="M311" s="2"/>
       <c r="N311" s="2"/>
@@ -11738,16 +12688,36 @@
     </row>
     <row r="312" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A312" s="2"/>
-      <c r="B312" s="2"/>
-      <c r="C312" s="2"/>
-      <c r="D312" s="2"/>
-      <c r="E312" s="2"/>
-      <c r="F312" s="2"/>
-      <c r="G312" s="2"/>
-      <c r="H312" s="2"/>
-      <c r="I312" s="2"/>
-      <c r="J312" s="2"/>
-      <c r="K312" s="2"/>
+      <c r="B312" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C312" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D312" s="19">
+        <v>83</v>
+      </c>
+      <c r="E312" s="19">
+        <v>51.55</v>
+      </c>
+      <c r="F312" s="19">
+        <v>84</v>
+      </c>
+      <c r="G312" s="19">
+        <v>8634370</v>
+      </c>
+      <c r="H312" s="19">
+        <v>43.77</v>
+      </c>
+      <c r="I312" s="19">
+        <v>5.33</v>
+      </c>
+      <c r="J312" s="19">
+        <v>1.07</v>
+      </c>
+      <c r="K312" s="19">
+        <v>108809.16</v>
+      </c>
       <c r="L312" s="2"/>
       <c r="M312" s="2"/>
       <c r="N312" s="2"/>
@@ -11766,16 +12736,36 @@
     </row>
     <row r="313" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A313" s="2"/>
-      <c r="B313" s="2"/>
-      <c r="C313" s="2"/>
-      <c r="D313" s="2"/>
-      <c r="E313" s="2"/>
-      <c r="F313" s="2"/>
-      <c r="G313" s="2"/>
-      <c r="H313" s="2"/>
-      <c r="I313" s="2"/>
-      <c r="J313" s="2"/>
-      <c r="K313" s="2"/>
+      <c r="B313" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C313" s="19" t="s">
+        <v>116</v>
+      </c>
+      <c r="D313" s="19">
+        <v>10</v>
+      </c>
+      <c r="E313" s="19">
+        <v>8.1999999999999993</v>
+      </c>
+      <c r="F313" s="19">
+        <v>10</v>
+      </c>
+      <c r="G313" s="19">
+        <v>1914496</v>
+      </c>
+      <c r="H313" s="19">
+        <v>12.84</v>
+      </c>
+      <c r="I313" s="19">
+        <v>2.5</v>
+      </c>
+      <c r="J313" s="19">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="K313" s="19">
+        <v>221401.60000000001</v>
+      </c>
       <c r="L313" s="2"/>
       <c r="M313" s="2"/>
       <c r="N313" s="2"/>
@@ -11794,16 +12784,36 @@
     </row>
     <row r="314" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A314" s="2"/>
-      <c r="B314" s="2"/>
-      <c r="C314" s="2"/>
-      <c r="D314" s="2"/>
-      <c r="E314" s="2"/>
-      <c r="F314" s="2"/>
-      <c r="G314" s="2"/>
-      <c r="H314" s="2"/>
-      <c r="I314" s="2"/>
-      <c r="J314" s="2"/>
-      <c r="K314" s="2"/>
+      <c r="B314" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C314" s="19" t="s">
+        <v>136</v>
+      </c>
+      <c r="D314" s="19">
+        <v>22</v>
+      </c>
+      <c r="E314" s="19">
+        <v>18.03</v>
+      </c>
+      <c r="F314" s="19">
+        <v>22</v>
+      </c>
+      <c r="G314" s="19">
+        <v>4933640</v>
+      </c>
+      <c r="H314" s="19">
+        <v>33.08</v>
+      </c>
+      <c r="I314" s="19">
+        <v>4.2300000000000004</v>
+      </c>
+      <c r="J314" s="19">
+        <v>1.1399999999999999</v>
+      </c>
+      <c r="K314" s="19">
+        <v>241245.68</v>
+      </c>
       <c r="L314" s="2"/>
       <c r="M314" s="2"/>
       <c r="N314" s="2"/>
@@ -11822,16 +12832,36 @@
     </row>
     <row r="315" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A315" s="2"/>
-      <c r="B315" s="2"/>
-      <c r="C315" s="2"/>
-      <c r="D315" s="2"/>
-      <c r="E315" s="2"/>
-      <c r="F315" s="2"/>
-      <c r="G315" s="2"/>
-      <c r="H315" s="2"/>
-      <c r="I315" s="2"/>
-      <c r="J315" s="2"/>
-      <c r="K315" s="2"/>
+      <c r="B315" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C315" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D315" s="19">
+        <v>34</v>
+      </c>
+      <c r="E315" s="19">
+        <v>27.87</v>
+      </c>
+      <c r="F315" s="19">
+        <v>34</v>
+      </c>
+      <c r="G315" s="19">
+        <v>3117182</v>
+      </c>
+      <c r="H315" s="19">
+        <v>20.9</v>
+      </c>
+      <c r="I315" s="19">
+        <v>3.26</v>
+      </c>
+      <c r="J315" s="19">
+        <v>1</v>
+      </c>
+      <c r="K315" s="19">
+        <v>91681.82</v>
+      </c>
       <c r="L315" s="2"/>
       <c r="M315" s="2"/>
       <c r="N315" s="2"/>
@@ -11850,16 +12880,36 @@
     </row>
     <row r="316" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A316" s="2"/>
-      <c r="B316" s="2"/>
-      <c r="C316" s="2"/>
-      <c r="D316" s="2"/>
-      <c r="E316" s="2"/>
-      <c r="F316" s="2"/>
-      <c r="G316" s="2"/>
-      <c r="H316" s="2"/>
-      <c r="I316" s="2"/>
-      <c r="J316" s="2"/>
-      <c r="K316" s="2"/>
+      <c r="B316" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C316" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="D316" s="19">
+        <v>56</v>
+      </c>
+      <c r="E316" s="19">
+        <v>45.9</v>
+      </c>
+      <c r="F316" s="19">
+        <v>56</v>
+      </c>
+      <c r="G316" s="19">
+        <v>4947673</v>
+      </c>
+      <c r="H316" s="19">
+        <v>33.18</v>
+      </c>
+      <c r="I316" s="19">
+        <v>5.54</v>
+      </c>
+      <c r="J316" s="19">
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="K316" s="19">
+        <v>96185.5</v>
+      </c>
       <c r="L316" s="2"/>
       <c r="M316" s="2"/>
       <c r="N316" s="2"/>
@@ -11878,16 +12928,16 @@
     </row>
     <row r="317" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A317" s="2"/>
-      <c r="B317" s="2"/>
-      <c r="C317" s="2"/>
-      <c r="D317" s="2"/>
-      <c r="E317" s="2"/>
-      <c r="F317" s="2"/>
-      <c r="G317" s="2"/>
-      <c r="H317" s="2"/>
-      <c r="I317" s="2"/>
-      <c r="J317" s="2"/>
-      <c r="K317" s="2"/>
+      <c r="B317" s="18"/>
+      <c r="C317" s="19"/>
+      <c r="D317" s="19"/>
+      <c r="E317" s="19"/>
+      <c r="F317" s="19"/>
+      <c r="G317" s="19"/>
+      <c r="H317" s="19"/>
+      <c r="I317" s="19"/>
+      <c r="J317" s="19"/>
+      <c r="K317" s="19"/>
       <c r="L317" s="2"/>
       <c r="M317" s="2"/>
       <c r="N317" s="2"/>
@@ -11906,16 +12956,18 @@
     </row>
     <row r="318" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A318" s="2"/>
-      <c r="B318" s="2"/>
-      <c r="C318" s="2"/>
-      <c r="D318" s="2"/>
-      <c r="E318" s="2"/>
-      <c r="F318" s="2"/>
-      <c r="G318" s="2"/>
-      <c r="H318" s="2"/>
-      <c r="I318" s="2"/>
-      <c r="J318" s="2"/>
-      <c r="K318" s="2"/>
+      <c r="B318" s="26" t="s">
+        <v>183</v>
+      </c>
+      <c r="C318" s="26"/>
+      <c r="D318" s="26"/>
+      <c r="E318" s="26"/>
+      <c r="F318" s="26"/>
+      <c r="G318" s="26"/>
+      <c r="H318" s="26"/>
+      <c r="I318" s="26"/>
+      <c r="J318" s="26"/>
+      <c r="K318" s="26"/>
       <c r="L318" s="2"/>
       <c r="M318" s="2"/>
       <c r="N318" s="2"/>
@@ -11934,16 +12986,16 @@
     </row>
     <row r="319" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A319" s="2"/>
-      <c r="B319" s="2"/>
-      <c r="C319" s="2"/>
-      <c r="D319" s="2"/>
-      <c r="E319" s="2"/>
-      <c r="F319" s="2"/>
-      <c r="G319" s="2"/>
-      <c r="H319" s="2"/>
-      <c r="I319" s="2"/>
-      <c r="J319" s="2"/>
-      <c r="K319" s="2"/>
+      <c r="B319" s="18"/>
+      <c r="C319" s="19"/>
+      <c r="D319" s="19"/>
+      <c r="E319" s="19"/>
+      <c r="F319" s="19"/>
+      <c r="G319" s="19"/>
+      <c r="H319" s="19"/>
+      <c r="I319" s="19"/>
+      <c r="J319" s="19"/>
+      <c r="K319" s="19"/>
       <c r="L319" s="2"/>
       <c r="M319" s="2"/>
       <c r="N319" s="2"/>
@@ -11962,16 +13014,34 @@
     </row>
     <row r="320" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A320" s="2"/>
-      <c r="B320" s="2"/>
-      <c r="C320" s="2"/>
-      <c r="D320" s="2"/>
-      <c r="E320" s="2"/>
-      <c r="F320" s="2"/>
-      <c r="G320" s="2"/>
-      <c r="H320" s="2"/>
-      <c r="I320" s="2"/>
-      <c r="J320" s="2"/>
-      <c r="K320" s="2"/>
+      <c r="B320" s="17" t="s">
+        <v>143</v>
+      </c>
+      <c r="C320" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="D320" s="17" t="s">
+        <v>144</v>
+      </c>
+      <c r="E320" s="17" t="s">
+        <v>145</v>
+      </c>
+      <c r="F320" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="G320" s="17" t="s">
+        <v>150</v>
+      </c>
+      <c r="H320" s="17" t="s">
+        <v>151</v>
+      </c>
+      <c r="I320" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="J320" s="17" t="s">
+        <v>169</v>
+      </c>
+      <c r="K320" s="19"/>
       <c r="L320" s="2"/>
       <c r="M320" s="2"/>
       <c r="N320" s="2"/>
@@ -11990,16 +13060,34 @@
     </row>
     <row r="321" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A321" s="2"/>
-      <c r="B321" s="2"/>
-      <c r="C321" s="2"/>
-      <c r="D321" s="2"/>
-      <c r="E321" s="2"/>
-      <c r="F321" s="2"/>
-      <c r="G321" s="2"/>
-      <c r="H321" s="2"/>
-      <c r="I321" s="2"/>
-      <c r="J321" s="2"/>
-      <c r="K321" s="2"/>
+      <c r="B321" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C321" s="19">
+        <v>32</v>
+      </c>
+      <c r="D321" s="19">
+        <v>28</v>
+      </c>
+      <c r="E321" s="19">
+        <v>4</v>
+      </c>
+      <c r="F321" s="19">
+        <v>2795602</v>
+      </c>
+      <c r="G321" s="19">
+        <v>2413802</v>
+      </c>
+      <c r="H321" s="19">
+        <v>381800</v>
+      </c>
+      <c r="I321" s="19" t="s">
+        <v>170</v>
+      </c>
+      <c r="J321" s="19" t="s">
+        <v>171</v>
+      </c>
+      <c r="K321" s="19"/>
       <c r="L321" s="2"/>
       <c r="M321" s="2"/>
       <c r="N321" s="2"/>
@@ -12018,16 +13106,34 @@
     </row>
     <row r="322" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A322" s="2"/>
-      <c r="B322" s="2"/>
-      <c r="C322" s="2"/>
-      <c r="D322" s="2"/>
-      <c r="E322" s="2"/>
-      <c r="F322" s="2"/>
-      <c r="G322" s="2"/>
-      <c r="H322" s="2"/>
-      <c r="I322" s="2"/>
-      <c r="J322" s="2"/>
-      <c r="K322" s="2"/>
+      <c r="B322" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C322" s="19">
+        <v>30</v>
+      </c>
+      <c r="D322" s="19">
+        <v>28</v>
+      </c>
+      <c r="E322" s="19">
+        <v>2</v>
+      </c>
+      <c r="F322" s="19">
+        <v>3765263</v>
+      </c>
+      <c r="G322" s="19">
+        <v>3303124</v>
+      </c>
+      <c r="H322" s="19">
+        <v>462139</v>
+      </c>
+      <c r="I322" s="19" t="s">
+        <v>172</v>
+      </c>
+      <c r="J322" s="19" t="s">
+        <v>173</v>
+      </c>
+      <c r="K322" s="19"/>
       <c r="L322" s="2"/>
       <c r="M322" s="2"/>
       <c r="N322" s="2"/>
@@ -12046,16 +13152,34 @@
     </row>
     <row r="323" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A323" s="2"/>
-      <c r="B323" s="2"/>
-      <c r="C323" s="2"/>
-      <c r="D323" s="2"/>
-      <c r="E323" s="2"/>
-      <c r="F323" s="2"/>
-      <c r="G323" s="2"/>
-      <c r="H323" s="2"/>
-      <c r="I323" s="2"/>
-      <c r="J323" s="2"/>
-      <c r="K323" s="2"/>
+      <c r="B323" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C323" s="19">
+        <v>34</v>
+      </c>
+      <c r="D323" s="19">
+        <v>29</v>
+      </c>
+      <c r="E323" s="19">
+        <v>5</v>
+      </c>
+      <c r="F323" s="19">
+        <v>4785585</v>
+      </c>
+      <c r="G323" s="19">
+        <v>4169668</v>
+      </c>
+      <c r="H323" s="19">
+        <v>615917</v>
+      </c>
+      <c r="I323" s="19" t="s">
+        <v>174</v>
+      </c>
+      <c r="J323" s="19" t="s">
+        <v>175</v>
+      </c>
+      <c r="K323" s="19"/>
       <c r="L323" s="2"/>
       <c r="M323" s="2"/>
       <c r="N323" s="2"/>
@@ -12074,16 +13198,34 @@
     </row>
     <row r="324" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A324" s="2"/>
-      <c r="B324" s="2"/>
-      <c r="C324" s="2"/>
-      <c r="D324" s="2"/>
-      <c r="E324" s="2"/>
-      <c r="F324" s="2"/>
-      <c r="G324" s="2"/>
-      <c r="H324" s="2"/>
-      <c r="I324" s="2"/>
-      <c r="J324" s="2"/>
-      <c r="K324" s="2"/>
+      <c r="B324" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C324" s="19">
+        <v>13</v>
+      </c>
+      <c r="D324" s="19">
+        <v>12</v>
+      </c>
+      <c r="E324" s="19">
+        <v>1</v>
+      </c>
+      <c r="F324" s="19">
+        <v>1356170</v>
+      </c>
+      <c r="G324" s="19">
+        <v>1249710</v>
+      </c>
+      <c r="H324" s="19">
+        <v>106460</v>
+      </c>
+      <c r="I324" s="19" t="s">
+        <v>176</v>
+      </c>
+      <c r="J324" s="19" t="s">
+        <v>177</v>
+      </c>
+      <c r="K324" s="19"/>
       <c r="L324" s="2"/>
       <c r="M324" s="2"/>
       <c r="N324" s="2"/>
@@ -12102,16 +13244,34 @@
     </row>
     <row r="325" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A325" s="2"/>
-      <c r="B325" s="2"/>
-      <c r="C325" s="2"/>
-      <c r="D325" s="2"/>
-      <c r="E325" s="2"/>
-      <c r="F325" s="2"/>
-      <c r="G325" s="2"/>
-      <c r="H325" s="2"/>
-      <c r="I325" s="2"/>
-      <c r="J325" s="2"/>
-      <c r="K325" s="2"/>
+      <c r="B325" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C325" s="19">
+        <v>9</v>
+      </c>
+      <c r="D325" s="19">
+        <v>7</v>
+      </c>
+      <c r="E325" s="19">
+        <v>2</v>
+      </c>
+      <c r="F325" s="19">
+        <v>1838464</v>
+      </c>
+      <c r="G325" s="19">
+        <v>1282460</v>
+      </c>
+      <c r="H325" s="19">
+        <v>556004</v>
+      </c>
+      <c r="I325" s="19" t="s">
+        <v>178</v>
+      </c>
+      <c r="J325" s="19" t="s">
+        <v>179</v>
+      </c>
+      <c r="K325" s="19"/>
       <c r="L325" s="2"/>
       <c r="M325" s="2"/>
       <c r="N325" s="2"/>
@@ -12130,16 +13290,34 @@
     </row>
     <row r="326" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A326" s="2"/>
-      <c r="B326" s="2"/>
-      <c r="C326" s="2"/>
-      <c r="D326" s="2"/>
-      <c r="E326" s="2"/>
-      <c r="F326" s="2"/>
-      <c r="G326" s="2"/>
-      <c r="H326" s="2"/>
-      <c r="I326" s="2"/>
-      <c r="J326" s="2"/>
-      <c r="K326" s="2"/>
+      <c r="B326" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C326" s="19">
+        <v>4</v>
+      </c>
+      <c r="D326" s="19">
+        <v>3</v>
+      </c>
+      <c r="E326" s="19">
+        <v>1</v>
+      </c>
+      <c r="F326" s="19">
+        <v>371907</v>
+      </c>
+      <c r="G326" s="19">
+        <v>325267</v>
+      </c>
+      <c r="H326" s="19">
+        <v>46640</v>
+      </c>
+      <c r="I326" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="J326" s="19" t="s">
+        <v>181</v>
+      </c>
+      <c r="K326" s="19"/>
       <c r="L326" s="2"/>
       <c r="M326" s="2"/>
       <c r="N326" s="2"/>
@@ -12158,16 +13336,34 @@
     </row>
     <row r="327" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A327" s="2"/>
-      <c r="B327" s="2"/>
-      <c r="C327" s="2"/>
-      <c r="D327" s="2"/>
-      <c r="E327" s="2"/>
-      <c r="F327" s="2"/>
-      <c r="G327" s="2"/>
-      <c r="H327" s="2"/>
-      <c r="I327" s="2"/>
-      <c r="J327" s="2"/>
-      <c r="K327" s="2"/>
+      <c r="B327" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C327" s="19">
+        <v>0</v>
+      </c>
+      <c r="D327" s="19">
+        <v>0</v>
+      </c>
+      <c r="E327" s="19">
+        <v>0</v>
+      </c>
+      <c r="F327" s="19">
+        <v>0</v>
+      </c>
+      <c r="G327" s="19">
+        <v>0</v>
+      </c>
+      <c r="H327" s="19">
+        <v>0</v>
+      </c>
+      <c r="I327" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="J327" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="K327" s="19"/>
       <c r="L327" s="2"/>
       <c r="M327" s="2"/>
       <c r="N327" s="2"/>
@@ -12186,16 +13382,16 @@
     </row>
     <row r="328" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A328" s="2"/>
-      <c r="B328" s="2"/>
-      <c r="C328" s="2"/>
-      <c r="D328" s="2"/>
-      <c r="E328" s="2"/>
-      <c r="F328" s="2"/>
-      <c r="G328" s="2"/>
-      <c r="H328" s="2"/>
-      <c r="I328" s="2"/>
-      <c r="J328" s="2"/>
-      <c r="K328" s="2"/>
+      <c r="B328" s="18"/>
+      <c r="C328" s="19"/>
+      <c r="D328" s="19"/>
+      <c r="E328" s="19"/>
+      <c r="F328" s="19"/>
+      <c r="G328" s="19"/>
+      <c r="H328" s="19"/>
+      <c r="I328" s="19"/>
+      <c r="J328" s="19"/>
+      <c r="K328" s="19"/>
       <c r="L328" s="2"/>
       <c r="M328" s="2"/>
       <c r="N328" s="2"/>
@@ -12214,16 +13410,6 @@
     </row>
     <row r="329" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A329" s="2"/>
-      <c r="B329" s="2"/>
-      <c r="C329" s="2"/>
-      <c r="D329" s="2"/>
-      <c r="E329" s="2"/>
-      <c r="F329" s="2"/>
-      <c r="G329" s="2"/>
-      <c r="H329" s="2"/>
-      <c r="I329" s="2"/>
-      <c r="J329" s="2"/>
-      <c r="K329" s="2"/>
       <c r="L329" s="2"/>
       <c r="M329" s="2"/>
       <c r="N329" s="2"/>
@@ -12242,16 +13428,18 @@
     </row>
     <row r="330" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A330" s="2"/>
-      <c r="B330" s="2"/>
-      <c r="C330" s="2"/>
-      <c r="D330" s="2"/>
-      <c r="E330" s="2"/>
-      <c r="F330" s="2"/>
-      <c r="G330" s="2"/>
-      <c r="H330" s="2"/>
-      <c r="I330" s="2"/>
-      <c r="J330" s="2"/>
-      <c r="K330" s="2"/>
+      <c r="B330" s="26" t="s">
+        <v>184</v>
+      </c>
+      <c r="C330" s="26"/>
+      <c r="D330" s="26"/>
+      <c r="E330" s="26"/>
+      <c r="F330" s="26"/>
+      <c r="G330" s="26"/>
+      <c r="H330" s="26"/>
+      <c r="I330" s="26"/>
+      <c r="J330" s="26"/>
+      <c r="K330" s="26"/>
       <c r="L330" s="2"/>
       <c r="M330" s="2"/>
       <c r="N330" s="2"/>
@@ -12270,16 +13458,26 @@
     </row>
     <row r="331" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A331" s="2"/>
-      <c r="B331" s="2"/>
-      <c r="C331" s="2"/>
-      <c r="D331" s="2"/>
-      <c r="E331" s="2"/>
-      <c r="F331" s="2"/>
-      <c r="G331" s="2"/>
-      <c r="H331" s="2"/>
-      <c r="I331" s="2"/>
-      <c r="J331" s="2"/>
-      <c r="K331" s="2"/>
+      <c r="B331" s="17" t="s">
+        <v>167</v>
+      </c>
+      <c r="C331" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="D331" s="17" t="s">
+        <v>146</v>
+      </c>
+      <c r="E331" s="17" t="s">
+        <v>152</v>
+      </c>
+      <c r="F331" s="17" t="s">
+        <v>185</v>
+      </c>
+      <c r="G331" s="19"/>
+      <c r="H331" s="19"/>
+      <c r="I331" s="19"/>
+      <c r="J331" s="19"/>
+      <c r="K331" s="19"/>
       <c r="L331" s="2"/>
       <c r="M331" s="2"/>
       <c r="N331" s="2"/>
@@ -12298,16 +13496,26 @@
     </row>
     <row r="332" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A332" s="2"/>
-      <c r="B332" s="2"/>
-      <c r="C332" s="2"/>
-      <c r="D332" s="2"/>
-      <c r="E332" s="2"/>
-      <c r="F332" s="2"/>
-      <c r="G332" s="2"/>
-      <c r="H332" s="2"/>
-      <c r="I332" s="2"/>
-      <c r="J332" s="2"/>
-      <c r="K332" s="2"/>
+      <c r="B332" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C332" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D332" s="19">
+        <v>0</v>
+      </c>
+      <c r="E332" s="19">
+        <v>0</v>
+      </c>
+      <c r="F332" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G332" s="19"/>
+      <c r="H332" s="19"/>
+      <c r="I332" s="19"/>
+      <c r="J332" s="19"/>
+      <c r="K332" s="19"/>
       <c r="L332" s="2"/>
       <c r="M332" s="2"/>
       <c r="N332" s="2"/>
@@ -12326,16 +13534,26 @@
     </row>
     <row r="333" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A333" s="2"/>
-      <c r="B333" s="2"/>
-      <c r="C333" s="2"/>
-      <c r="D333" s="2"/>
-      <c r="E333" s="2"/>
-      <c r="F333" s="2"/>
-      <c r="G333" s="2"/>
-      <c r="H333" s="2"/>
-      <c r="I333" s="2"/>
-      <c r="J333" s="2"/>
-      <c r="K333" s="2"/>
+      <c r="B333" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C333" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D333" s="19">
+        <v>12</v>
+      </c>
+      <c r="E333" s="19">
+        <v>1829710</v>
+      </c>
+      <c r="F333" s="19" t="s">
+        <v>188</v>
+      </c>
+      <c r="G333" s="19"/>
+      <c r="H333" s="19"/>
+      <c r="I333" s="19"/>
+      <c r="J333" s="19"/>
+      <c r="K333" s="19"/>
       <c r="L333" s="2"/>
       <c r="M333" s="2"/>
       <c r="N333" s="2"/>
@@ -12354,16 +13572,26 @@
     </row>
     <row r="334" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A334" s="2"/>
-      <c r="B334" s="2"/>
-      <c r="C334" s="2"/>
-      <c r="D334" s="2"/>
-      <c r="E334" s="2"/>
-      <c r="F334" s="2"/>
-      <c r="G334" s="2"/>
-      <c r="H334" s="2"/>
-      <c r="I334" s="2"/>
-      <c r="J334" s="2"/>
-      <c r="K334" s="2"/>
+      <c r="B334" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C334" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D334" s="19">
+        <v>12</v>
+      </c>
+      <c r="E334" s="19">
+        <v>441447</v>
+      </c>
+      <c r="F334" s="19" t="s">
+        <v>189</v>
+      </c>
+      <c r="G334" s="19"/>
+      <c r="H334" s="19"/>
+      <c r="I334" s="19"/>
+      <c r="J334" s="19"/>
+      <c r="K334" s="19"/>
       <c r="L334" s="2"/>
       <c r="M334" s="2"/>
       <c r="N334" s="2"/>
@@ -12382,16 +13610,26 @@
     </row>
     <row r="335" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A335" s="2"/>
-      <c r="B335" s="2"/>
-      <c r="C335" s="2"/>
-      <c r="D335" s="2"/>
-      <c r="E335" s="2"/>
-      <c r="F335" s="2"/>
-      <c r="G335" s="2"/>
-      <c r="H335" s="2"/>
-      <c r="I335" s="2"/>
-      <c r="J335" s="2"/>
-      <c r="K335" s="2"/>
+      <c r="B335" s="18">
+        <v>46230</v>
+      </c>
+      <c r="C335" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D335" s="19">
+        <v>8</v>
+      </c>
+      <c r="E335" s="19">
+        <v>524445</v>
+      </c>
+      <c r="F335" s="19" t="s">
+        <v>191</v>
+      </c>
+      <c r="G335" s="19"/>
+      <c r="H335" s="19"/>
+      <c r="I335" s="19"/>
+      <c r="J335" s="19"/>
+      <c r="K335" s="19"/>
       <c r="L335" s="2"/>
       <c r="M335" s="2"/>
       <c r="N335" s="2"/>
@@ -12410,16 +13648,26 @@
     </row>
     <row r="336" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A336" s="2"/>
-      <c r="B336" s="2"/>
-      <c r="C336" s="2"/>
-      <c r="D336" s="2"/>
-      <c r="E336" s="2"/>
-      <c r="F336" s="2"/>
-      <c r="G336" s="2"/>
-      <c r="H336" s="2"/>
-      <c r="I336" s="2"/>
-      <c r="J336" s="2"/>
-      <c r="K336" s="2"/>
+      <c r="B336" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C336" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D336" s="19">
+        <v>0</v>
+      </c>
+      <c r="E336" s="19">
+        <v>0</v>
+      </c>
+      <c r="F336" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G336" s="19"/>
+      <c r="H336" s="19"/>
+      <c r="I336" s="19"/>
+      <c r="J336" s="19"/>
+      <c r="K336" s="19"/>
       <c r="L336" s="2"/>
       <c r="M336" s="2"/>
       <c r="N336" s="2"/>
@@ -12438,16 +13686,26 @@
     </row>
     <row r="337" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A337" s="2"/>
-      <c r="B337" s="2"/>
-      <c r="C337" s="2"/>
-      <c r="D337" s="2"/>
-      <c r="E337" s="2"/>
-      <c r="F337" s="2"/>
-      <c r="G337" s="2"/>
-      <c r="H337" s="2"/>
-      <c r="I337" s="2"/>
-      <c r="J337" s="2"/>
-      <c r="K337" s="2"/>
+      <c r="B337" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C337" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D337" s="19">
+        <v>12</v>
+      </c>
+      <c r="E337" s="19">
+        <v>2374338</v>
+      </c>
+      <c r="F337" s="19" t="s">
+        <v>192</v>
+      </c>
+      <c r="G337" s="19"/>
+      <c r="H337" s="19"/>
+      <c r="I337" s="19"/>
+      <c r="J337" s="19"/>
+      <c r="K337" s="19"/>
       <c r="L337" s="2"/>
       <c r="M337" s="2"/>
       <c r="N337" s="2"/>
@@ -12466,16 +13724,26 @@
     </row>
     <row r="338" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A338" s="2"/>
-      <c r="B338" s="2"/>
-      <c r="C338" s="2"/>
-      <c r="D338" s="2"/>
-      <c r="E338" s="2"/>
-      <c r="F338" s="2"/>
-      <c r="G338" s="2"/>
-      <c r="H338" s="2"/>
-      <c r="I338" s="2"/>
-      <c r="J338" s="2"/>
-      <c r="K338" s="2"/>
+      <c r="B338" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C338" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D338" s="19">
+        <v>12</v>
+      </c>
+      <c r="E338" s="19">
+        <v>744822</v>
+      </c>
+      <c r="F338" s="19" t="s">
+        <v>193</v>
+      </c>
+      <c r="G338" s="19"/>
+      <c r="H338" s="19"/>
+      <c r="I338" s="19"/>
+      <c r="J338" s="19"/>
+      <c r="K338" s="19"/>
       <c r="L338" s="2"/>
       <c r="M338" s="2"/>
       <c r="N338" s="2"/>
@@ -12494,16 +13762,26 @@
     </row>
     <row r="339" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A339" s="2"/>
-      <c r="B339" s="2"/>
-      <c r="C339" s="2"/>
-      <c r="D339" s="2"/>
-      <c r="E339" s="2"/>
-      <c r="F339" s="2"/>
-      <c r="G339" s="2"/>
-      <c r="H339" s="2"/>
-      <c r="I339" s="2"/>
-      <c r="J339" s="2"/>
-      <c r="K339" s="2"/>
+      <c r="B339" s="18">
+        <v>46231</v>
+      </c>
+      <c r="C339" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D339" s="19">
+        <v>6</v>
+      </c>
+      <c r="E339" s="19">
+        <v>646103</v>
+      </c>
+      <c r="F339" s="19" t="s">
+        <v>194</v>
+      </c>
+      <c r="G339" s="19"/>
+      <c r="H339" s="19"/>
+      <c r="I339" s="19"/>
+      <c r="J339" s="19"/>
+      <c r="K339" s="19"/>
       <c r="L339" s="2"/>
       <c r="M339" s="2"/>
       <c r="N339" s="2"/>
@@ -12522,16 +13800,26 @@
     </row>
     <row r="340" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A340" s="2"/>
-      <c r="B340" s="2"/>
-      <c r="C340" s="2"/>
-      <c r="D340" s="2"/>
-      <c r="E340" s="2"/>
-      <c r="F340" s="2"/>
-      <c r="G340" s="2"/>
-      <c r="H340" s="2"/>
-      <c r="I340" s="2"/>
-      <c r="J340" s="2"/>
-      <c r="K340" s="2"/>
+      <c r="B340" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C340" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D340" s="19">
+        <v>0</v>
+      </c>
+      <c r="E340" s="19">
+        <v>0</v>
+      </c>
+      <c r="F340" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G340" s="19"/>
+      <c r="H340" s="19"/>
+      <c r="I340" s="19"/>
+      <c r="J340" s="19"/>
+      <c r="K340" s="19"/>
       <c r="L340" s="2"/>
       <c r="M340" s="2"/>
       <c r="N340" s="2"/>
@@ -12550,16 +13838,26 @@
     </row>
     <row r="341" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A341" s="2"/>
-      <c r="B341" s="2"/>
-      <c r="C341" s="2"/>
-      <c r="D341" s="2"/>
-      <c r="E341" s="2"/>
-      <c r="F341" s="2"/>
-      <c r="G341" s="2"/>
-      <c r="H341" s="2"/>
-      <c r="I341" s="2"/>
-      <c r="J341" s="2"/>
-      <c r="K341" s="2"/>
+      <c r="B341" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C341" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D341" s="19">
+        <v>13</v>
+      </c>
+      <c r="E341" s="19">
+        <v>3417644</v>
+      </c>
+      <c r="F341" s="19" t="s">
+        <v>195</v>
+      </c>
+      <c r="G341" s="19"/>
+      <c r="H341" s="19"/>
+      <c r="I341" s="19"/>
+      <c r="J341" s="19"/>
+      <c r="K341" s="19"/>
       <c r="L341" s="2"/>
       <c r="M341" s="2"/>
       <c r="N341" s="2"/>
@@ -12578,16 +13876,26 @@
     </row>
     <row r="342" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A342" s="2"/>
-      <c r="B342" s="2"/>
-      <c r="C342" s="2"/>
-      <c r="D342" s="2"/>
-      <c r="E342" s="2"/>
-      <c r="F342" s="2"/>
-      <c r="G342" s="2"/>
-      <c r="H342" s="2"/>
-      <c r="I342" s="2"/>
-      <c r="J342" s="2"/>
-      <c r="K342" s="2"/>
+      <c r="B342" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C342" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D342" s="19">
+        <v>9</v>
+      </c>
+      <c r="E342" s="19">
+        <v>351664</v>
+      </c>
+      <c r="F342" s="19" t="s">
+        <v>196</v>
+      </c>
+      <c r="G342" s="19"/>
+      <c r="H342" s="19"/>
+      <c r="I342" s="19"/>
+      <c r="J342" s="19"/>
+      <c r="K342" s="19"/>
       <c r="L342" s="2"/>
       <c r="M342" s="2"/>
       <c r="N342" s="2"/>
@@ -12606,16 +13914,26 @@
     </row>
     <row r="343" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A343" s="2"/>
-      <c r="B343" s="2"/>
-      <c r="C343" s="2"/>
-      <c r="D343" s="2"/>
-      <c r="E343" s="2"/>
-      <c r="F343" s="2"/>
-      <c r="G343" s="2"/>
-      <c r="H343" s="2"/>
-      <c r="I343" s="2"/>
-      <c r="J343" s="2"/>
-      <c r="K343" s="2"/>
+      <c r="B343" s="18">
+        <v>46232</v>
+      </c>
+      <c r="C343" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D343" s="19">
+        <v>12</v>
+      </c>
+      <c r="E343" s="19">
+        <v>1016277</v>
+      </c>
+      <c r="F343" s="19" t="s">
+        <v>197</v>
+      </c>
+      <c r="G343" s="19"/>
+      <c r="H343" s="19"/>
+      <c r="I343" s="19"/>
+      <c r="J343" s="19"/>
+      <c r="K343" s="19"/>
       <c r="L343" s="2"/>
       <c r="M343" s="2"/>
       <c r="N343" s="2"/>
@@ -12634,16 +13952,26 @@
     </row>
     <row r="344" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A344" s="2"/>
-      <c r="B344" s="2"/>
-      <c r="C344" s="2"/>
-      <c r="D344" s="2"/>
-      <c r="E344" s="2"/>
-      <c r="F344" s="2"/>
-      <c r="G344" s="2"/>
-      <c r="H344" s="2"/>
-      <c r="I344" s="2"/>
-      <c r="J344" s="2"/>
-      <c r="K344" s="2"/>
+      <c r="B344" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C344" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D344" s="19">
+        <v>0</v>
+      </c>
+      <c r="E344" s="19">
+        <v>0</v>
+      </c>
+      <c r="F344" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G344" s="19"/>
+      <c r="H344" s="19"/>
+      <c r="I344" s="19"/>
+      <c r="J344" s="19"/>
+      <c r="K344" s="19"/>
       <c r="L344" s="2"/>
       <c r="M344" s="2"/>
       <c r="N344" s="2"/>
@@ -12662,16 +13990,26 @@
     </row>
     <row r="345" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A345" s="2"/>
-      <c r="B345" s="2"/>
-      <c r="C345" s="2"/>
-      <c r="D345" s="2"/>
-      <c r="E345" s="2"/>
-      <c r="F345" s="2"/>
-      <c r="G345" s="2"/>
-      <c r="H345" s="2"/>
-      <c r="I345" s="2"/>
-      <c r="J345" s="2"/>
-      <c r="K345" s="2"/>
+      <c r="B345" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C345" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D345" s="19">
+        <v>4</v>
+      </c>
+      <c r="E345" s="19">
+        <v>711558</v>
+      </c>
+      <c r="F345" s="19" t="s">
+        <v>198</v>
+      </c>
+      <c r="G345" s="19"/>
+      <c r="H345" s="19"/>
+      <c r="I345" s="19"/>
+      <c r="J345" s="19"/>
+      <c r="K345" s="19"/>
       <c r="L345" s="2"/>
       <c r="M345" s="2"/>
       <c r="N345" s="2"/>
@@ -12690,16 +14028,26 @@
     </row>
     <row r="346" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A346" s="2"/>
-      <c r="B346" s="2"/>
-      <c r="C346" s="2"/>
-      <c r="D346" s="2"/>
-      <c r="E346" s="2"/>
-      <c r="F346" s="2"/>
-      <c r="G346" s="2"/>
-      <c r="H346" s="2"/>
-      <c r="I346" s="2"/>
-      <c r="J346" s="2"/>
-      <c r="K346" s="2"/>
+      <c r="B346" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C346" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D346" s="19">
+        <v>6</v>
+      </c>
+      <c r="E346" s="19">
+        <v>362612</v>
+      </c>
+      <c r="F346" s="19" t="s">
+        <v>199</v>
+      </c>
+      <c r="G346" s="19"/>
+      <c r="H346" s="19"/>
+      <c r="I346" s="19"/>
+      <c r="J346" s="19"/>
+      <c r="K346" s="19"/>
       <c r="L346" s="2"/>
       <c r="M346" s="2"/>
       <c r="N346" s="2"/>
@@ -12718,16 +14066,26 @@
     </row>
     <row r="347" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A347" s="2"/>
-      <c r="B347" s="2"/>
-      <c r="C347" s="2"/>
-      <c r="D347" s="2"/>
-      <c r="E347" s="2"/>
-      <c r="F347" s="2"/>
-      <c r="G347" s="2"/>
-      <c r="H347" s="2"/>
-      <c r="I347" s="2"/>
-      <c r="J347" s="2"/>
-      <c r="K347" s="2"/>
+      <c r="B347" s="18">
+        <v>46233</v>
+      </c>
+      <c r="C347" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D347" s="19">
+        <v>3</v>
+      </c>
+      <c r="E347" s="19">
+        <v>282000</v>
+      </c>
+      <c r="F347" s="19" t="s">
+        <v>200</v>
+      </c>
+      <c r="G347" s="19"/>
+      <c r="H347" s="19"/>
+      <c r="I347" s="19"/>
+      <c r="J347" s="19"/>
+      <c r="K347" s="19"/>
       <c r="L347" s="2"/>
       <c r="M347" s="2"/>
       <c r="N347" s="2"/>
@@ -12746,16 +14104,26 @@
     </row>
     <row r="348" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A348" s="2"/>
-      <c r="B348" s="2"/>
-      <c r="C348" s="2"/>
-      <c r="D348" s="2"/>
-      <c r="E348" s="2"/>
-      <c r="F348" s="2"/>
-      <c r="G348" s="2"/>
-      <c r="H348" s="2"/>
-      <c r="I348" s="2"/>
-      <c r="J348" s="2"/>
-      <c r="K348" s="2"/>
+      <c r="B348" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C348" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D348" s="19">
+        <v>0</v>
+      </c>
+      <c r="E348" s="19">
+        <v>0</v>
+      </c>
+      <c r="F348" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G348" s="19"/>
+      <c r="H348" s="19"/>
+      <c r="I348" s="19"/>
+      <c r="J348" s="19"/>
+      <c r="K348" s="19"/>
       <c r="L348" s="2"/>
       <c r="M348" s="2"/>
       <c r="N348" s="2"/>
@@ -12774,16 +14142,26 @@
     </row>
     <row r="349" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A349" s="2"/>
-      <c r="B349" s="2"/>
-      <c r="C349" s="2"/>
-      <c r="D349" s="2"/>
-      <c r="E349" s="2"/>
-      <c r="F349" s="2"/>
-      <c r="G349" s="2"/>
-      <c r="H349" s="2"/>
-      <c r="I349" s="2"/>
-      <c r="J349" s="2"/>
-      <c r="K349" s="2"/>
+      <c r="B349" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C349" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D349" s="19">
+        <v>3</v>
+      </c>
+      <c r="E349" s="19">
+        <v>959318</v>
+      </c>
+      <c r="F349" s="19" t="s">
+        <v>201</v>
+      </c>
+      <c r="G349" s="19"/>
+      <c r="H349" s="19"/>
+      <c r="I349" s="19"/>
+      <c r="J349" s="19"/>
+      <c r="K349" s="19"/>
       <c r="L349" s="2"/>
       <c r="M349" s="2"/>
       <c r="N349" s="2"/>
@@ -12802,16 +14180,26 @@
     </row>
     <row r="350" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A350" s="2"/>
-      <c r="B350" s="2"/>
-      <c r="C350" s="2"/>
-      <c r="D350" s="2"/>
-      <c r="E350" s="2"/>
-      <c r="F350" s="2"/>
-      <c r="G350" s="2"/>
-      <c r="H350" s="2"/>
-      <c r="I350" s="2"/>
-      <c r="J350" s="2"/>
-      <c r="K350" s="2"/>
+      <c r="B350" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C350" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D350" s="19">
+        <v>4</v>
+      </c>
+      <c r="E350" s="19">
+        <v>413886</v>
+      </c>
+      <c r="F350" s="19" t="s">
+        <v>202</v>
+      </c>
+      <c r="G350" s="19"/>
+      <c r="H350" s="19"/>
+      <c r="I350" s="19"/>
+      <c r="J350" s="19"/>
+      <c r="K350" s="19"/>
       <c r="L350" s="2"/>
       <c r="M350" s="2"/>
       <c r="N350" s="2"/>
@@ -12830,16 +14218,26 @@
     </row>
     <row r="351" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A351" s="2"/>
-      <c r="B351" s="2"/>
-      <c r="C351" s="2"/>
-      <c r="D351" s="2"/>
-      <c r="E351" s="2"/>
-      <c r="F351" s="2"/>
-      <c r="G351" s="2"/>
-      <c r="H351" s="2"/>
-      <c r="I351" s="2"/>
-      <c r="J351" s="2"/>
-      <c r="K351" s="2"/>
+      <c r="B351" s="18">
+        <v>46234</v>
+      </c>
+      <c r="C351" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D351" s="19">
+        <v>2</v>
+      </c>
+      <c r="E351" s="19">
+        <v>465260</v>
+      </c>
+      <c r="F351" s="19" t="s">
+        <v>203</v>
+      </c>
+      <c r="G351" s="19"/>
+      <c r="H351" s="19"/>
+      <c r="I351" s="19"/>
+      <c r="J351" s="19"/>
+      <c r="K351" s="19"/>
       <c r="L351" s="2"/>
       <c r="M351" s="2"/>
       <c r="N351" s="2"/>
@@ -12858,16 +14256,26 @@
     </row>
     <row r="352" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A352" s="2"/>
-      <c r="B352" s="2"/>
-      <c r="C352" s="2"/>
-      <c r="D352" s="2"/>
-      <c r="E352" s="2"/>
-      <c r="F352" s="2"/>
-      <c r="G352" s="2"/>
-      <c r="H352" s="2"/>
-      <c r="I352" s="2"/>
-      <c r="J352" s="2"/>
-      <c r="K352" s="2"/>
+      <c r="B352" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C352" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D352" s="19">
+        <v>0</v>
+      </c>
+      <c r="E352" s="19">
+        <v>0</v>
+      </c>
+      <c r="F352" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G352" s="19"/>
+      <c r="H352" s="19"/>
+      <c r="I352" s="19"/>
+      <c r="J352" s="19"/>
+      <c r="K352" s="19"/>
       <c r="L352" s="2"/>
       <c r="M352" s="2"/>
       <c r="N352" s="2"/>
@@ -12886,16 +14294,26 @@
     </row>
     <row r="353" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A353" s="2"/>
-      <c r="B353" s="2"/>
-      <c r="C353" s="2"/>
-      <c r="D353" s="2"/>
-      <c r="E353" s="2"/>
-      <c r="F353" s="2"/>
-      <c r="G353" s="2"/>
-      <c r="H353" s="2"/>
-      <c r="I353" s="2"/>
-      <c r="J353" s="2"/>
-      <c r="K353" s="2"/>
+      <c r="B353" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C353" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D353" s="19">
+        <v>1</v>
+      </c>
+      <c r="E353" s="19">
+        <v>153917</v>
+      </c>
+      <c r="F353" s="19" t="s">
+        <v>204</v>
+      </c>
+      <c r="G353" s="19"/>
+      <c r="H353" s="19"/>
+      <c r="I353" s="19"/>
+      <c r="J353" s="19"/>
+      <c r="K353" s="19"/>
       <c r="L353" s="2"/>
       <c r="M353" s="2"/>
       <c r="N353" s="2"/>
@@ -12914,16 +14332,26 @@
     </row>
     <row r="354" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A354" s="2"/>
-      <c r="B354" s="2"/>
-      <c r="C354" s="2"/>
-      <c r="D354" s="2"/>
-      <c r="E354" s="2"/>
-      <c r="F354" s="2"/>
-      <c r="G354" s="2"/>
-      <c r="H354" s="2"/>
-      <c r="I354" s="2"/>
-      <c r="J354" s="2"/>
-      <c r="K354" s="2"/>
+      <c r="B354" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C354" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D354" s="19">
+        <v>2</v>
+      </c>
+      <c r="E354" s="19">
+        <v>126550</v>
+      </c>
+      <c r="F354" s="19" t="s">
+        <v>205</v>
+      </c>
+      <c r="G354" s="19"/>
+      <c r="H354" s="19"/>
+      <c r="I354" s="19"/>
+      <c r="J354" s="19"/>
+      <c r="K354" s="19"/>
       <c r="L354" s="2"/>
       <c r="M354" s="2"/>
       <c r="N354" s="2"/>
@@ -12942,16 +14370,26 @@
     </row>
     <row r="355" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A355" s="2"/>
-      <c r="B355" s="2"/>
-      <c r="C355" s="2"/>
-      <c r="D355" s="2"/>
-      <c r="E355" s="2"/>
-      <c r="F355" s="2"/>
-      <c r="G355" s="2"/>
-      <c r="H355" s="2"/>
-      <c r="I355" s="2"/>
-      <c r="J355" s="2"/>
-      <c r="K355" s="2"/>
+      <c r="B355" s="18">
+        <v>46235</v>
+      </c>
+      <c r="C355" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D355" s="19">
+        <v>1</v>
+      </c>
+      <c r="E355" s="19">
+        <v>91440</v>
+      </c>
+      <c r="F355" s="19" t="s">
+        <v>206</v>
+      </c>
+      <c r="G355" s="19"/>
+      <c r="H355" s="19"/>
+      <c r="I355" s="19"/>
+      <c r="J355" s="19"/>
+      <c r="K355" s="19"/>
       <c r="L355" s="2"/>
       <c r="M355" s="2"/>
       <c r="N355" s="2"/>
@@ -12970,16 +14408,26 @@
     </row>
     <row r="356" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A356" s="2"/>
-      <c r="B356" s="2"/>
-      <c r="C356" s="2"/>
-      <c r="D356" s="2"/>
-      <c r="E356" s="2"/>
-      <c r="F356" s="2"/>
-      <c r="G356" s="2"/>
-      <c r="H356" s="2"/>
-      <c r="I356" s="2"/>
-      <c r="J356" s="2"/>
-      <c r="K356" s="2"/>
+      <c r="B356" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C356" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="D356" s="19">
+        <v>0</v>
+      </c>
+      <c r="E356" s="19">
+        <v>0</v>
+      </c>
+      <c r="F356" s="19" t="s">
+        <v>182</v>
+      </c>
+      <c r="G356" s="19"/>
+      <c r="H356" s="19"/>
+      <c r="I356" s="19"/>
+      <c r="J356" s="19"/>
+      <c r="K356" s="19"/>
       <c r="L356" s="2"/>
       <c r="M356" s="2"/>
       <c r="N356" s="2"/>
@@ -12998,11 +14446,21 @@
     </row>
     <row r="357" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A357" s="2"/>
-      <c r="B357" s="2"/>
-      <c r="C357" s="2"/>
-      <c r="D357" s="2"/>
-      <c r="E357" s="2"/>
-      <c r="F357" s="2"/>
+      <c r="B357" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C357" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D357" s="19">
+        <v>0</v>
+      </c>
+      <c r="E357" s="19">
+        <v>0</v>
+      </c>
+      <c r="F357" s="19" t="s">
+        <v>182</v>
+      </c>
       <c r="G357" s="2"/>
       <c r="H357" s="2"/>
       <c r="I357" s="2"/>
@@ -13026,11 +14484,21 @@
     </row>
     <row r="358" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A358" s="2"/>
-      <c r="B358" s="2"/>
-      <c r="C358" s="2"/>
-      <c r="D358" s="2"/>
-      <c r="E358" s="2"/>
-      <c r="F358" s="2"/>
+      <c r="B358" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C358" s="19" t="s">
+        <v>165</v>
+      </c>
+      <c r="D358" s="19">
+        <v>0</v>
+      </c>
+      <c r="E358" s="19">
+        <v>0</v>
+      </c>
+      <c r="F358" s="19" t="s">
+        <v>182</v>
+      </c>
       <c r="G358" s="2"/>
       <c r="H358" s="2"/>
       <c r="I358" s="2"/>
@@ -13054,11 +14522,21 @@
     </row>
     <row r="359" spans="1:26" ht="13" x14ac:dyDescent="0.15">
       <c r="A359" s="2"/>
-      <c r="B359" s="2"/>
-      <c r="C359" s="2"/>
-      <c r="D359" s="2"/>
-      <c r="E359" s="2"/>
-      <c r="F359" s="2"/>
+      <c r="B359" s="18">
+        <v>46236</v>
+      </c>
+      <c r="C359" s="19" t="s">
+        <v>190</v>
+      </c>
+      <c r="D359" s="19">
+        <v>0</v>
+      </c>
+      <c r="E359" s="19">
+        <v>0</v>
+      </c>
+      <c r="F359" s="19" t="s">
+        <v>182</v>
+      </c>
       <c r="G359" s="2"/>
       <c r="H359" s="2"/>
       <c r="I359" s="2"/>
@@ -31196,13 +32674,38 @@
       <c r="Y1006" s="2"/>
       <c r="Z1006" s="2"/>
     </row>
+    <row r="1007" spans="1:26" ht="13" x14ac:dyDescent="0.15">
+      <c r="A1007" s="2"/>
+      <c r="B1007" s="2"/>
+      <c r="C1007" s="2"/>
+      <c r="D1007" s="2"/>
+      <c r="E1007" s="2"/>
+      <c r="F1007" s="2"/>
+      <c r="G1007" s="2"/>
+      <c r="H1007" s="2"/>
+      <c r="I1007" s="2"/>
+      <c r="J1007" s="2"/>
+      <c r="K1007" s="2"/>
+      <c r="L1007" s="2"/>
+      <c r="M1007" s="2"/>
+      <c r="N1007" s="2"/>
+      <c r="O1007" s="2"/>
+      <c r="P1007" s="2"/>
+      <c r="Q1007" s="2"/>
+      <c r="R1007" s="2"/>
+      <c r="S1007" s="2"/>
+      <c r="T1007" s="2"/>
+      <c r="U1007" s="2"/>
+      <c r="V1007" s="2"/>
+      <c r="W1007" s="2"/>
+      <c r="X1007" s="2"/>
+      <c r="Y1007" s="2"/>
+      <c r="Z1007" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="12">
-    <mergeCell ref="B256:G256"/>
-    <mergeCell ref="A83:C83"/>
-    <mergeCell ref="A97:C97"/>
-    <mergeCell ref="A106:G106"/>
-    <mergeCell ref="A129:G129"/>
+  <mergeCells count="17">
+    <mergeCell ref="B318:K318"/>
+    <mergeCell ref="B330:K330"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A5:C5"/>
@@ -31210,6 +32713,14 @@
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A30:C30"/>
     <mergeCell ref="A74:C74"/>
+    <mergeCell ref="B264:K264"/>
+    <mergeCell ref="B274:F274"/>
+    <mergeCell ref="B287:K287"/>
+    <mergeCell ref="B256:G256"/>
+    <mergeCell ref="A83:C83"/>
+    <mergeCell ref="A97:C97"/>
+    <mergeCell ref="A106:G106"/>
+    <mergeCell ref="A129:G129"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>

</xml_diff>